<commit_message>
save 03 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_26_Cursor.xlsx
+++ b/4 четверть_26_Cursor.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DFD80E0-B4EE-4BB9-A415-C4D8AB810C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BD2ECE-84B2-4A2B-9C84-0AD102BE32FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2310" yWindow="-15720" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Основные настройки" sheetId="1" r:id="rId1"/>
     <sheet name="Активный функционал" sheetId="2" r:id="rId2"/>
     <sheet name="Template" sheetId="3" r:id="rId3"/>
+    <sheet name="Prompts" sheetId="4" r:id="rId4"/>
+    <sheet name="Не программирование Prompts" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="451">
   <si>
     <t>Настройки Cursor</t>
   </si>
@@ -2203,17 +2205,1868 @@
     <t>1 Выведи список библиотек/зависимостей с версиями из @package.json 
 2 отсортируй список dependencies (production) от наиболее часто используемых библиотек к наименее в проекте</t>
   </si>
+  <si>
+    <t>{
+  "hooks": {
+    "beforeShellExecution": [
+      {
+        "type": "prompt",
+        "prompt": "Проанализируй следующую команду консоли/оболочки (shell) на безопасность. \nСТРОГИЕ ПРАВИЛА:\n1. БАЗА ДАННЫХ: Разрешены ИСКЛЮЧИТЕЛЬНО операции чтения (SELECT) напрямую или через вызов .sql файлов. Запрещены любые изменения БД (INSERT, UPDATE, DELETE, DROP, ALTER, TRUNCATE).\n2. СКРИПТЫ: Запрещено исполнение непроверенных скриптов (.sh, .py, .js, .pl), если они могут изменять систему или БД. Разрешены только строго read-only скрипты.\n3. ФАЙЛОВАЯ СИСТЕМА И ОС: Запрещены деструктивные команды (rm -rf, dd, mkfs, перезапись системных файлов, &gt; /dev/sda). Запрещены опасные изменения прав (chmod 777, chown). Разрешены только команды чтения и навигации (ls, cat, find, grep, head, tail, cd, pwd).\n4. СЕТЬ И ЭКСПЛУАТАЦИЯ: Запрещены произвольные исходящие сетевые запросы (curl, wget, nc, ssh), если они не являются частью безопасного read-only API. Запрещена эксфильтрация данных.\n5. УПРАВЛЕНИЕ СИСТЕМОЙ: Запрещены команды управления процессами и службами (kill, pkill, reboot, shutdown, systemctl, service).\n6. МЕНЕДЖЕРЫ ПАКЕТОВ: Запрещена установка или обновление пакетов (apt, yum, pip, npm install), кроме случаев, когда это явно требуется для read-only задачи.\nОтветь СТРОГО в формате JSON: {\"allow\": true/false, \"reason\": \"краткое объяснение\"}",
+        "timeout": 15
+      }
+    ],
+    "beforeFileWrite": [
+      {
+        "type": "prompt",
+        "prompt": "Проанализируй содержимое файла, который агент пытается записать на диск.\nПРАВИЛА:\n1. Если это исполняемый скрипт (.sh, .py, .js), запрети запись, если он содержит команды изменения БД, удаления файлов (rm) или сетевые запросы.\n2. Запрети запись в системные директории (/etc, /bin, /usr) и скрытые конфигурационные файлы (~/.bashrc, ~/.ssh).\nОтветь СТРОГО в формате JSON: {\"allow\": true/false, \"reason\": \"краткое объяснение\"}",
+        "timeout": 15
+      }
+    ],
+    "beforeFileRead": [
+      {
+        "type": "prompt",
+        "prompt": "Проанализируй запрос на чтение файла. Запрети чтение файлов, содержащих конфиденциальные данные (пароли, токены, .env, приватные ключи, ~/.ssh/*), если это не требуется для текущей read-only задачи. Ответь JSON: {\"allow\": true/false, \"reason\": \"...\"}",
+        "timeout": 10
+      }
+    ]
+  }
+}</t>
+  </si>
+  <si>
+    <t>`https://loops.elorm.xyz/loops</t>
+  </si>
+  <si>
+    <t>Библиотека промптов</t>
+  </si>
+  <si>
+    <t>Ресурсы с промптами</t>
+  </si>
+  <si>
+    <t>Start the "Investigation Script Loop" loop.
+Goal: prove the root cause with a minimal repro script
+Max iterations: 8
+Between iterations run: node scripts/investigate.mjs
+Exit when: script output demonstrates root cause
+Step 1: Write a tiny throwaway script that reproduces the issue. Run it and iterate on what the output shows.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Debugging</t>
+  </si>
+  <si>
+    <t>Поиск бага, но не разрешение проблемы</t>
+  </si>
+  <si>
+    <t>Start the "Reflexion Debug Loop" loop.
+Goal: the failing test or repro passes
+Max iterations: 8
+Between iterations run: npm test -- --testNamePattern=&lt;failing-test&gt;
+Exit when: the repro test exits 0
+Step 1: Reproduce the bug. If it fails, append a reflection to .loops/reflexion.md before trying a new fix.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Исправление бага</t>
+  </si>
+  <si>
+    <t>Start the "Guardrails Learning Loop" loop.
+Goal: tests and lint pass without repeating prior failure patterns
+Max iterations: 12
+Between iterations run: npm test &amp;&amp; npm run lint
+Exit when: all checks pass
+Step 1: Read .ralph/guardrails.md, run checks, and if a failure repeats, add a sign before fixing.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Исключение паттернов исправлений, которые привели к ошибке ранее</t>
+  </si>
+  <si>
+    <t>Выполнение после планирования</t>
+  </si>
+  <si>
+    <t>в отдельном файле</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Start the "Ralph Story Executor" loop.
+Goal: every story in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.ralph/prd.json</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> has passes: true
+Max iterations: 20
+Between iterations run: npm test &amp;&amp; npm run lint &amp;&amp; npm run build
+Exit when: no stories remain with passes: false (respond "ALL STORIES ARE COMPLETE")
+Step 1: Read .ralph/prd.json and .ralph/progress.md. Pick one incomplete story, implement it, run backpressure checks, commit, update prd.json and progress.md, then stop this iteration.
+Self-pace this loop. Each iteration does exactly one story. State lives on disk, not in chat history.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Start the "OpenAPI Sync Until Valid" loop.
+Goal: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>openapi.yaml</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> lints clean and matches implemented routes
+Max iterations: 8
+Between iterations run: npx @redocly/cli lint openapi.yaml
+Exit when: OpenAPI lint exits 0
+Step 1: Lint openapi.yaml. Fix spec errors and handler drift until lint passes.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Выполнение ранее спланированных задач (+ тесты), содержащихся </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>в файле</t>
+    </r>
+  </si>
+  <si>
+    <t>Start the "API Contract Until Match" loop.
+Goal: API implementation matches the published contract
+Max iterations: 10
+Between iterations run: npm run test:contract
+Exit when: contract test suite exits 0
+Step 1: Run contract tests. Fix each schema/response mismatch with minimal diffs, then re-run.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Создание/проверка интеграционной спецификации</t>
+  </si>
+  <si>
+    <t>Проверка/исправление контрактов (интеграционное тестирование)</t>
+  </si>
+  <si>
+    <t>Start the "Ship PR Until Green" loop.
+Goal: PR is open with all CI checks passing
+Max iterations: 10
+Between iterations run: gh pr checks
+Exit when: all PR checks are success
+Step 1: Implement the change, test locally, push, open PR, and fix CI until green.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>CI/CD</t>
+  </si>
+  <si>
+    <t>/loop 5m Start the "CI Failure Watcher" loop.
+Goal: latest CI run on this branch is green.
+Max iterations: 12.
+Between iterations run: gh run list --branch $(git branch --show-current) --limit 1
+Exit when: latest run conclusion is success.
+Step 1: Check CI status. If failed, read logs, fix root cause, verify locally, and push if needed.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>/loop 15m Start the "PR Watch Loop".
+Goal: keep codex-watch PRs healthy and unblocked.
+Between iterations run: gh pr list --label codex-watch --json number,title,state,statusCheckRollup
+Exit when: status report is delivered for every watched PR.
+Step 1: List codex-watch PRs, check CI and reviews, and report or fix trivial blockers.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>/loop 15m Start the "PR Babysitter" loop.
+Goal: open PRs labeled codex-watch are healthy (CI green, rebased, not stale).
+Max iterations: 20.
+Between iterations run: gh pr list --label "codex-watch"
+Exit when: each watched PR is green and current, or escalated.
+Step 1: List watched PRs. Fix CI once, rebase if behind, comment if stale. Escalate repeated failures.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Start the "Fix CI Until Green" loop.
+Goal: latest CI run on this branch passes
+Max iterations: 8
+Between iterations run: gh run list --branch $(git branch --show-current) --limit 1 --json conclusion -q '.[0].conclusion'
+Exit when: latest run conclusion is success
+Step 1: Find the latest failed CI run, read logs, reproduce locally, fix root cause, push, and verify.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Для Senior</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1) чтение и вывод статистики по открытым PR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Для Senior</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1) чтение и вывод статистики по открытым PR
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2)исправление ошибок</t>
+    </r>
+  </si>
+  <si>
+    <t>2 (оптимальнее №1)</t>
+  </si>
+  <si>
+    <t>3 (оптимальнее №2)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1 PR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Когда план выполнен, запустить чтобы проверить/исправить написанный код, протестировать его, запушить в </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">gitlab (любую указанную платформу по контролю версий), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>добиться чтобы все тесты, сборка стали зелеными</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Multiple PR</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1) Позволяет получать дашборд с описанием открытых PR под тэгом codex watched и статусами по каждому из них.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Multiple PR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1) Позволяет получать дашборд с описанием открытых PR под тэгом codex watched и статусами по каждому из них.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2) Агент не просто наблюдает и докладывает, а активно вмешивается и заботится о здоровье PR</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1 PR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Когда план выполнен, запустить чтобы проверить/исправить написанный код, протестировать его, запушить в </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">gitlab (любую указанную платформу по контролю версий), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>добиться чтобы все тесты, сборка стали зелеными</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Отличие от №1:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> работает более низкоуровнево с gitlab ci, проверяя заключения пайплайнов и джобов по отдельности, затем исправляя ошибки в коде и отправляя новый коммит. Также предусмотрен механизм ожидания отработки pipeline (5 минут) - меньше тратится токенов и меньше запросов к gitlab</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1 PR
+Отличие от №2: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1 Он сам должен "само-paced" (self-pace) регулировать темп — то есть понимать, что после git push новый CI-ран ещё не завершился, и не спамить GitHub API запросами</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2 Команда gh run list --branch $(git branch --show-current) --limit 1 --json conclusion -q '.[0].conclusion' — это значительное улучшение по сравнению с обычным gh run list: Агенту не нужно парсить табличный вывод с колонками — он получает чистое значение, которое легко сравнить с success
+3 Reproduce locally — критически важный шаг! Агент должен попытаться воспроизвести ошибку локально перед тем, как её чинить. Это предотвращает "слепой фикс" — когда агент меняет код наугад, надеясь, что CI пройдёт.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>Start the "Migration Until Applied" loop.
+Goal: all database migrations apply cleanly
+Max iterations: 6
+Between iterations run: npx prisma migrate status
+Exit when: migrate status shows no pending failures
+Step 1: Run migrations. Fix schema or SQL errors, then repeat until status is clean.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2) Команда npx prisma migrate status — это специфичный инструмент Prisma, который показывает:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 Применённые миграции
+2 Ожидающие (pending) миграции
+3 Drift — расхождение между схемой в БД и schema.prisma
+4 Ошибки применения</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Недостатки промпта:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 Нет запрета на деструктивные операции (DROP, DELETE без WHERE)
+2 Нет требования делать бэкап перед применением
+3 Нет упоминания о migrate dev --create-only для безопасного создания миграций
+4 Нет проверки на наличие данных в таблицах перед изменением схемы</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1) Агент работает с базой данных, где операции могут быть:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 Деструктивными (DROP TABLE, удаление колонок с данными)
+2 Необратимыми (потеря данных при неправильной миграции)
+3 Зависящими от состояния (миграция может пройти на пустой БД, но упасть на заполненной)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Это делает данный промпт наиболее рискованным из всей серии.</t>
+    </r>
+  </si>
+  <si>
+    <t>Стартовые промпты</t>
+  </si>
+  <si>
+    <t>1 Проиндексировать проект, используя https://dev.to/arshtechpro/stop-making-your-ai-coding-agent-grep-your-whole-repo-try-codebase-memory-mcp-4g8l
+2 Создать файл endpoints.json, где будут описаны все endpoint сервера, а также их контракты
+3 Создать правило стягивать ветку test, создавать test_sergeev если нет, обновлять test_sergeev к test, обновить структуру в файле endpoints.json? а затем выполнять очередной prompt</t>
+  </si>
+  <si>
+    <t>Deploy</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Миграция базы данных</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 Автоматической генерации миграций (например, после изменения schema.prisma другим агентом)
+2 Разрешении конфликтов миграций в команде
+3 Восстановлении состояния БД после сбоев</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">/loop 15m Start the "Deploy Verification Loop".
+Goal: all post-deploy health and smoke endpoints return success.
+Max iterations: 8.
+Between iterations run: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>curl -fsS &lt;your-health-url&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Exit when: every configured endpoint succeeds.
+Step 1: Hit health/smoke URLs. If any fail, inspect deploy logs and fix or escalate.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>После запуска проекта на сервере будет запущен цикл</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, который окончится когда все endpoints вернут success. Цикл будет проверять на health каждый endpoint, указанный в списке endpoints
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Например
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://api.example.com/health
+https://api.example.com/healthz
+https://api.example.com/readyz</t>
+    </r>
+  </si>
+  <si>
+    <t>Start the "Changelog Sync After Ship" loop.
+Goal: CHANGELOG.md has accurate [Unreleased] entries for this ship
+Max iterations: 3
+Between iterations run: git log -5 --oneline
+Exit when: changelog covers all user-visible changes
+Step 1: Review recent commits, write Keep-a-Changelog entries for user-visible changes, and verify completeness.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Создание документации изменений для внешних пользователей</t>
+  </si>
+  <si>
+    <t>Before starting:
+- Run `git fetch origin main` to get latest changes
+- Check `git status` to understand current state
+- Verify you're on the correct branch
+During rebase:
+- Resolve conflicts one file at a time
+- After each file, run `grep -r "&lt;&lt;&lt;&lt;&lt;&lt;&lt; HEAD" . || echo "No conflicts"` to verify
+- For package-lock.json/yarn.lock: accept main version and run `npm install`
+- For binary files: escalate immediately (don't attempt to resolve)
+- For migrations: escalate if uncertain about semantics
+After rebase:
+- Run `git status` to verify rebase is complete
+- Run `npm test` to verify tests pass
+- If tests fail, check if it's due to your resolution or pre-existing issue
+- If due to your resolution, fix and re-test
+- If pre-existing, adapt your code to work with main changes
+Escape hatch:
+- If more than 5 conflicts or complex semantic conflicts, escalate instead of continuing
+- Use `git rebase --abort` only if rebase is completely broken</t>
+  </si>
+  <si>
+    <t>Git</t>
+  </si>
+  <si>
+    <r>
+      <t>Разрешение rebase conflict 
+с т</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">екущей ветки </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+к ветке </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>main</t>
+    </r>
+  </si>
+  <si>
+    <t>1 Создание документации изменений для внешних пользователей
+2 Полезно для передачи менеджерам
+3 Работает только с одним файлом (CHANGELOG.md),</t>
+  </si>
+  <si>
+    <t>Правило!</t>
+  </si>
+  <si>
+    <t>Всегда используй максимальную reasoning модели на стадии планирования. На стадии исполнения плана можно использовать средний уровень reasoning.</t>
+  </si>
+  <si>
+    <t>Создание внутренней документации изменений</t>
+  </si>
+  <si>
+    <t>Start the "Docs Sync After Edits" loop.
+Goal: documentation matches the current code changes
+Max iterations: 3
+Between iterations run: git diff main...HEAD --name-only
+Exit when: all affected docs are updated and verified
+Step 1: Review the diff, find stale docs, update them, and verify accuracy.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Коммит будет задокументирован в API, inline комментах</t>
+  </si>
+  <si>
+    <t>Обновление зависимостей в проекте (еженедельно)</t>
+  </si>
+  <si>
+    <t>/loop 7d Start the "Dependency Audit Weekly" loop.
+Goal: deliver a weekly dependency audit summary.
+Between iterations run: npm outdated || true
+Exit when: summary is posted with recommended upgrades.
+Step 1: Run npm outdated, categorize updates, and propose a safe upgrade plan.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Before starting:
+- Verify Knip is configured correctly (knip.json exists)
+- Understand project type (app/library/monorepo)
+- Run `npx knip --include exports` to see what will be checked
+During cleanup:
+- Remove unused dependencies first (safest)
+- Then remove unused files
+- Then remove unused exports (most risky)
+- After each removal, run `npm test` AND `npm run build`
+- For libraries, check if export is part of public API before removing
+Escape hatch:
+- If Knip reports "possibly unused", escalate instead of removing
+- If removing breaks tests, revert and investigate
+- If more than 20 items to remove, split into multiple PRs</t>
+  </si>
+  <si>
+    <t>Удаление мертвых зависимостей</t>
+  </si>
+  <si>
+    <t>Start the "Knip Until Clean" loop.
+Goal: knip reports no unused code or dependencies
+Max iterations: 5
+Between iterations run: npx knip
+Exit when: knip exits 0
+Step 1: Run knip. Remove dead exports and unused deps with minimal diffs; verify tests still pass.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Start the "Dependency Upgrade One-by-One" loop.
+Goal: critical outdated deps are upgraded with green tests
+Max iterations: 15
+Between iterations run: npm outdated &amp;&amp; npm test &amp;&amp; npm run build
+Exit when: npm outdated shows no critical packages left or user stops
+Step 1: Pick one outdated package, upgrade it, fix breakages, commit, and stop. One package per iteration.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Обновляет зависимости</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1 Проверяет зависимости на outdated и составляет план обновлений.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2 Не обновляет самостоятельно</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+3 Каждые 7 дней</t>
+    </r>
+  </si>
+  <si>
+    <t>/loop 7d Start the "Security Audit Weekly" loop.
+Goal: deliver a weekly npm audit summary with a remediation plan.
+Between iterations run: npm audit --json
+Exit when: summary is posted with prioritized fixes.
+Step 1: Run npm audit, triage by severity, and propose safe remediation steps.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1 Проверяет зависимости на vulnerabilities и составляет план обновлений.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">2 Не обновляет самостоятельно
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3 Каждые 7 дней</t>
+    </r>
+  </si>
+  <si>
+    <t>Когнитивно сложная задача</t>
+  </si>
+  <si>
+    <t>Start the "Bundle Size Budget" loop.
+Goal: client bundle stays under the size-limit budget
+Max iterations: 6
+Between iterations run: npm run build &amp;&amp; npm run size-limit
+Exit when: size-limit exits 0
+Step 1: Build and measure bundle size. If over budget, lazy-load or trim deps until size-limit passes.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Сокращение размера package/build</t>
+  </si>
+  <si>
+    <t>Планирование</t>
+  </si>
+  <si>
+    <t>Ведение истории багов и решений</t>
+  </si>
+  <si>
+    <t>/using-superpowers используя субагент, напиши спецификацию (spec.md) для реализации подхода 2 со всеми требованиями и нюансами к проекту, очень развернуто прописывая этапы перевода graphql на rest (этап - это перевод с graphql на rest одного backend endpoint и соответствующего frontend fetch запроса). Тебе нужно учесть, нюансы moleculer и vue composition api фреймворков. В каждом этапе пропиши необходимые юнит тесты и интеграционные тесты. Пропиши, что любое тестирование не должно касаться базы данных. Тестируй только выполнение запросов между front и back исключая дальнейшие вызовы к базе данных.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/using-superpowers - Я собираюсь переписать проект с graphql на rest. Пройди по этим шагам: Шаг 1: сформулируй, что именно я решаю. Шаг 2: назови три альтернативных подхода. Шаг 3: для каждого — плюсы, минусы, когда подходит. Шаг 4: дай рекомендацию с обоснованием. Не пропускай шаги, не объединяй их. </t>
+  </si>
+  <si>
+    <t>Запрос 1</t>
+  </si>
+  <si>
+    <t>Запрос 2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Routes всего проекта</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Если есть swagger.json содержащий все параметры, которые ожидают обработчики на сервере, а также ответы, то можно запустить интеграционное тестирование, сославшись на такой </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>json файл</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Routes всего проекта</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Тестирование/создание файла swagger.json, который содержит всю информацию об обработчиках на сервере, чтобы потом использовать его как эталон при внесении изменений на front и back</t>
+    </r>
+  </si>
+  <si>
+    <t>Интеграционные тесты</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Routes внесенных изменений</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Start the "Spec-First Ship" loop.
+Goal: every requirement in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>spec.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is implemented and checked off
+Max iterations: 15
+Between iterations run: npm test
+Exit when: spec.md has no unchecked requirements
+Step 1: Read spec.md, implement the first unchecked item, verify it, mark [x], and stop this iteration.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+    </r>
+  </si>
+  <si>
+    <t>Start the "A11y Audit Until Clean" loop.
+Goal: zero serious accessibility violations on changed UI
+Max iterations: 8
+Between iterations run: npm run test:a11y
+Exit when: a11y audit exits 0
+Step 1: Run the a11y audit on changed routes. Fix each violation, prioritizing keyboard and screen reader issues.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Code review</t>
+  </si>
+  <si>
+    <t>По внесенным изменениям</t>
+  </si>
+  <si>
+    <t>Start the "PR Self-Review" loop.
+Goal: PR passes all automated checks and has no critical manual findings
+Max iterations: 3
+Between iterations run:
+  1. npm run lint
+  2. npm run typecheck
+  3. npm test
+  4. npm audit
+  5. git diff main...HEAD (for manual review)
+Exit when: all automated checks pass AND manual review finds no critical issues
+Step 1: Run all automated checks. Fix any failures.
+Step 2: Manual review pass 1 - correctness (logic, edge cases, error handling)
+Step 3: Manual review pass 2 - security &amp; performance
+Step 4: Manual review pass 3 - readability &amp; maintainability
+Step 5: Document all findings and their status
+Critical findings (must fix):
+- Security vulnerabilities
+- Data loss risks
+- Breaking changes to public API
+- Missing error handling in critical paths
+- Race conditions
+Non-critical findings (should fix):
+- Code style issues
+- Suboptimal naming
+- Missing comments
+Guardrails (do not skip):
+- Do not consider a pass "clean" if automated checks fail
+- Do not ignore findings from previous passes
+- Do not disable checks to pass
+- If stuck after several iterations, stop and report blockers</t>
+  </si>
+  <si>
+    <t>Start the "PR Self-Review" loop.
+Goal: three clean self-review passes on the current diff
+Max iterations: 3
+Between iterations run: git diff main...HEAD
+Exit when: three passes complete with no critical findings
+Step 1: Review the diff like a senior reviewer. Fix findings, then re-review.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Оптимизация синтаксиса проекта</t>
+  </si>
+  <si>
+    <t>Before starting:
+- Run `npm run lint` to catch style issues
+- Run `grep` commands to find debug artifacts:
+  - `grep -rn "console\." src/ --include="*.ts"`
+  - `grep -rn "debugger" src/`
+  - `grep -rn "TODO\|FIXME\|HACK" src/`
+- Understand project conventions (naming, structure, patterns)
+De-sloppify checklist:
+Pass 1: Debug artifacts
+- Remove console.log/debug/info (except explicit error handlers)
+- Remove debugger statements
+- Remove temporary variables
+- Remove commented-out debug code
+Pass 2: Dead code
+- Remove commented-out code blocks (unless TODO with context)
+- Remove unreachable code (after return/throw)
+- Remove empty catch blocks (add proper error handling)
+- Remove useless else after return
+- Remove unused parameters (prefix with _ if needed)
+Pass 3: Naming &amp; style
+- Fix names to follow project conventions
+- Replace meaningless names (data, result, temp)
+- Fix incorrect abbreviations
+- Replace magic numbers with constants
+- Keep comments that explain WHY, remove comments that explain WHAT
+After each change:
+- Run `npm run lint &amp;&amp; npm test`
+- Verify code is not worse after cleanup
+- Use minimal diffs (one logical change at a time)
+Escape hatch:
+- If unsure whether something is slop, escalate
+- If removing breaks tests, revert and investigate
+- If more than 4 iterations needed, reassess approach</t>
+  </si>
+  <si>
+    <t>Start the "De-Sloppify Pass" loop.
+Goal: recent changes are clean, minimal, and convention-aligned
+Max iterations: 4
+Between iterations run: npm run lint &amp;&amp; npm test
+Exit when: review finds no slop and checks pass
+Step 1: Review the diff for debug code, dead branches, and naming issues. Fix them with minimal diffs.
+Self-pace this loop. After each iteration, run the check command, read the output, and only continue if the exit condition is not met. Stop when the exit condition passes or max iterations is reached. Give a short status update each pass.
+Guardrails (do not skip):
+- Do not modify the check command or exit criteria to force success
+- Do not skip, disable, or bypass checks to pass the exit condition
+- If stuck after several iterations, stop and report blockers instead of gaming metrics</t>
+  </si>
+  <si>
+    <t>Caveman skill/plugin</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">`https://github.com/juliusbrussee/caveman
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Install (using bash):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> curl -fsSL https://raw.githubusercontent.com/JuliusBrussee/caveman/main/install.sh | bash
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Remove:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> npx -y github:JuliusBrussee/caveman -- --uninstall
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Trigger:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> type /caveman or say "talk like caveman". 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Stop</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with "normal mode".</t>
+    </r>
+  </si>
+  <si>
+    <t>/caveman [lite|full|ultra|wenyan]	Compress every reply. Levels stick until session end.
+/caveman-commit	Conventional Commit messages, ≤50 char subject. Why over what.
+/caveman-review	One-line PR comments: L42: 🔴 bug: user null. Add guard.
+/caveman-stats	Real session token usage + lifetime savings + USD. Tweetable line via --share.
+/caveman-compress &lt;file&gt;	Rewrite memory file (e.g. CLAUDE.md) into caveman-speak. Cuts ~46% input tokens every session. Code/URLs/paths byte-preserved.
+caveman-shrink	MCP middleware. Wraps any MCP server, compresses tool descriptions. npm.
+cavecrew-*	Caveman subagents (investigator/builder/reviewer). ~60% fewer tokens than vanilla, main context lasts longer.</t>
+  </si>
+  <si>
+    <t>Библиотека скиллов</t>
+  </si>
+  <si>
+    <t>`https://github.com/JuliusBrussee/skills/blob/main/skills/fuck-slop/references/voices.md</t>
+  </si>
+  <si>
+    <t>context-canary</t>
+  </si>
+  <si>
+    <t>Когда вы работаете с AI-агентом в длинной сессии (особенно с такими циклами, как мы разбирали — loop-kit), происходит несколько незаметных процессов:
+Context rot — ранние инструкции из начала диалога (80k+ токенов назад) перестают учитываться моделью
+Compaction — система автоматически сжимает историю, и при сжатии теряются standing instructions (постоянные правила)
+Instruction drift — модель постепенно перестаёт следовать правилам, которые были заданы в начале
+Lost-in-the-middle — модель хуже всего "видит" информацию в середине длинного контекста</t>
+  </si>
+  <si>
+    <t>`https://github.com/JuliusBrussee/skills/blob/main/skills/context-canary/SKILL.md</t>
+  </si>
+  <si>
+    <t>`https://github.com/JuliusBrussee/skills/blob/main/skills/fuck-slop/SKILL.md</t>
+  </si>
+  <si>
+    <t>fuck-slop</t>
+  </si>
+  <si>
+    <t>Убирает напыщенная лексика из ответов и результатов ИИ</t>
+  </si>
+  <si>
+    <t>`https://github.com/JuliusBrussee/skills/blob/main/skills/interface-kit/SKILL.md</t>
+  </si>
+  <si>
+    <t>interface-kit</t>
+  </si>
+  <si>
+    <t>UI skill</t>
+  </si>
+  <si>
+    <t>`https://github.com/JuliusBrussee/skills/blob/main/skills/grill-me/SKILL.md</t>
+  </si>
+  <si>
+    <t>Задать вопросы пользователю по составленному плану</t>
+  </si>
+  <si>
+    <t>grill-me</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Junior-режим (дефолтное поведение LLM)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Реактивное выполнение:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Получил задачу → сразу начал писать код
+Не задал уточняющих вопросов
+Не подумал, почему эта задача вообще возникла
+Сделал буквально то, что попросили, даже если это плохое решение
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Отсутствие контекста:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Не учитывает legacy code, team conventions, business requirements
+Не понимает, что этот файл трогать нельзя (потому что его использует другой сервис)
+Не видит, что предлагаемое решение конфликтует с архитектурой проекта
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Нет trade-off анализа:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Предлагает одно решение без альтернатив
+Не объясняет, почему выбрал этот подход
+Не упоминает, какие у решения есть downsides
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Игнорирование последствий:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Не думает о том, что будет через месяц
+Не учитывает maintainability, scalability, security
+Не предвидит edge cases
+Не проверяет, не сломает ли это что-то ещё
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Страх эскалации:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Пытается "починить" всё сам, даже когда не понимает контекст
+Не говорит "я не уверен, нужно ли это делать"
+Не предлагает остановиться и обсудить</t>
+    </r>
+  </si>
+  <si>
+    <t>junior-to-senior</t>
+  </si>
+  <si>
+    <t>`https://github.com/JuliusBrussee/skills/tree/main/skills/junior-to-senior</t>
+  </si>
+  <si>
+    <t>`https://github.com/JuliusBrussee/skills/tree/main/skills/loop-factory</t>
+  </si>
+  <si>
+    <t>loop-factory</t>
+  </si>
+  <si>
+    <t>мониторинг: помнит ли агент, как думать</t>
+  </si>
+  <si>
+    <t>качество: удаление AI-артефактов из результатов</t>
+  </si>
+  <si>
+    <t>Создание новых циклов</t>
+  </si>
+  <si>
+    <t>Всегда использовать!</t>
+  </si>
+  <si>
+    <t>`https://github.com/mattpocock/skills/blob/main/skills/in-progress/wayfinder/SKILL.md</t>
+  </si>
+  <si>
+    <t>wayfinder</t>
+  </si>
+  <si>
+    <t>Позволяет создать файл, где зранятся все текущие и будущие вопрос по принципу fog of war</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Всегда использовать! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Планирование</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Всегда использовать! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ВСЕГДА</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Всегда использовать!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> UI</t>
+    </r>
+  </si>
+  <si>
+    <t>Использовать во всех ситуациях</t>
+  </si>
+  <si>
+    <t>Настойка CI/CD проекта:
+Копирование ключей и тд с bash скриптом и пошаговым ведением</t>
+  </si>
+  <si>
+    <t>`https://github.com/mattpocock/skills/blob/main/skills/in-progress/wizard/SKILL.md</t>
+  </si>
+  <si>
+    <t>wizard</t>
+  </si>
+  <si>
+    <t>writing-beats</t>
+  </si>
+  <si>
+    <t>`https://github.com/mattpocock/skills/tree/main/skills/in-progress/writing-beats</t>
+  </si>
+  <si>
+    <t>Написание статей</t>
+  </si>
+  <si>
+    <t>`https://github.com/mattpocock/skills/tree/main/skills/in-progress/writing-fragments</t>
+  </si>
+  <si>
+    <t>writing-fragments</t>
+  </si>
+  <si>
+    <t>Отвечает за хаотичный сбор идей</t>
+  </si>
+  <si>
+    <t>За выстраивание нарратива (истории)</t>
+  </si>
+  <si>
+    <t>`https://github.com/mattpocock/skills/blob/main/skills/in-progress/writing-shape/SKILL.md</t>
+  </si>
+  <si>
+    <t>writing-shape</t>
+  </si>
+  <si>
+    <t>Превращает груды сырого материала в логичную, структурированную статью, абзац за абзацем. гарантирует, что итоговый текст будет удобен для чтения</t>
+  </si>
+  <si>
+    <t>Behavioral guidelines to reduce common LLM coding mistakes. Merge with project-specific instructions as needed.
+Tradeoff: These guidelines bias toward caution over speed. For trivial tasks, use judgment.
+1. Think Before Coding
+Don't assume. Don't hide confusion. Surface tradeoffs.
+Before implementing:
+State your assumptions explicitly. If uncertain, ask.
+If multiple interpretations exist, present them - don't pick silently.
+If a simpler approach exists, say so. Push back when warranted.
+If something is unclear, stop. Name what's confusing. Ask.
+2. Simplicity First
+Minimum code that solves the problem. Nothing speculative.
+No features beyond what was asked.
+No abstractions for single-use code.
+No "flexibility" or "configurability" that wasn't requested.
+No error handling for impossible scenarios.
+If you write 200 lines and it could be 50, rewrite it.
+Ask yourself: "Would a senior engineer say this is overcomplicated?" If yes, simplify.
+3. Surgical Changes
+Touch only what you must. Clean up only your own mess.
+When editing existing code:
+Don't "improve" adjacent code, comments, or formatting.
+Don't refactor things that aren't broken.
+Match existing style, even if you'd do it differently.
+If you notice unrelated dead code, mention it - don't delete it.
+When your changes create orphans:
+Remove imports/variables/functions that YOUR changes made unused.
+Don't remove pre-existing dead code unless asked.
+The test: Every changed line should trace directly to the user's request.
+4. Goal-Driven Execution
+Define success criteria. Loop until verified.
+Transform tasks into verifiable goals:
+"Add validation" → "Write tests for invalid inputs, then make them pass"
+"Fix the bug" → "Write a test that reproduces it, then make it pass"
+"Refactor X" → "Ensure tests pass before and after"
+For multi-step tasks, state a brief plan:
+1. [Step] → verify: [check]
+2. [Step] → verify: [check]
+3. [Step] → verify: [check]
+Strong success criteria let you loop independently. Weak criteria ("make it work") require constant clarification.
+These guidelines are working if: fewer unnecessary changes in diffs, fewer rewrites due to overcomplication, and clarifying questions come before implementation rather than after mistakes.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2388,8 +4241,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2438,6 +4308,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2450,9 +4326,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2460,13 +4336,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -2476,7 +4352,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -2489,90 +4365,120 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5733,7 +7639,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:U55"/>
+  <dimension ref="A2:U60"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" style="1" customWidth="1"/>
@@ -5830,388 +7736,1244 @@
         <v>284</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
+        <v>355</v>
+      </c>
+      <c r="C12" s="35"/>
+    </row>
+    <row r="13" spans="1:21" s="21" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C13" s="43" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="C14" s="43"/>
+    </row>
+    <row r="15" spans="1:21" s="21" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" s="49" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="36"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="38"/>
-    </row>
-    <row r="13" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="35" t="s">
+      <c r="B16" s="36"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="38"/>
+    </row>
+    <row r="17" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="35" t="s">
         <v>274</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B17" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C17" s="42" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B14" s="21" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B18" s="21" t="s">
         <v>269</v>
       </c>
-      <c r="C14" s="42" t="s">
+      <c r="C18" s="42" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="64.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21" t="s">
+    <row r="19" spans="1:4" ht="64.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="21" t="s">
         <v>271</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="C19" s="35" t="s">
         <v>278</v>
       </c>
-      <c r="D15" s="35" t="s">
+      <c r="D19" s="35" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="35" t="s">
+    <row r="20" spans="1:4" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="35" t="s">
         <v>281</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D20" s="21" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B17" s="21" t="s">
+    <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B21" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C17" s="35" t="s">
+      <c r="C21" s="35" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="35" t="s">
+    <row r="23" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="35" t="s">
         <v>275</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="B23" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="C19" s="41" t="s">
+      <c r="C23" s="41" t="s">
         <v>313</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="21" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B24" s="21" t="s">
         <v>269</v>
       </c>
-      <c r="C20" s="41" t="s">
+      <c r="C24" s="41" t="s">
         <v>314</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="39" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B25" s="39" t="s">
         <v>291</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C25" s="31" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C22" s="16" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C26" s="16" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C24" s="41" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C28" s="41" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
+    <row r="29" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B29" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="C25" s="35"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
+      <c r="C29" s="35"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B30" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="C26" s="35"/>
-    </row>
-    <row r="27" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
+      <c r="C30" s="35"/>
+    </row>
+    <row r="31" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B27" s="35" t="s">
+      <c r="B31" s="35" t="s">
         <v>252</v>
       </c>
-      <c r="C27" s="35"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="39" t="s">
+      <c r="C31" s="35"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B32" s="39" t="s">
         <v>292</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C32" s="15" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
+    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B34" s="29" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="17" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B35" s="17" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="22" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B36" s="17" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="22" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B33" s="35" t="s">
+      <c r="B37" s="35" t="s">
         <v>294</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B34" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B35" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B36" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B37" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B38" s="34" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B39" s="40" t="s">
-        <v>67</v>
+      <c r="B39" s="24" t="s">
+        <v>59</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B40" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B41" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B42" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B43" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B44" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B41" s="24" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B45" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C45" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B42" s="21" t="s">
+    <row r="46" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B46" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="8" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="8" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A44" s="17" t="s">
+    <row r="48" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="B44" s="29" t="s">
+      <c r="B48" s="29" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="17" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="B45" s="21" t="s">
+      <c r="B49" s="21" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="22" t="s">
+    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B46" s="35" t="s">
+      <c r="B50" s="35" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="22" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B47" s="21" t="s">
+      <c r="B51" s="21" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="8" t="s">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="8" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="17" t="s">
+    <row r="53" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B53" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D53" s="1" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A50" s="17" t="s">
+    <row r="54" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A54" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="C50" s="35" t="s">
+      <c r="C54" s="35" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A51" s="22" t="s">
+    <row r="55" spans="1:4" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A55" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B55" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="C51" s="35" t="s">
+      <c r="C55" s="35" t="s">
         <v>307</v>
       </c>
-      <c r="D51" s="35" t="s">
+      <c r="D55" s="35" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="216" x14ac:dyDescent="0.3">
-      <c r="A52" s="22"/>
-      <c r="B52" s="17"/>
-      <c r="C52" s="35" t="s">
+    <row r="56" spans="1:4" ht="216" x14ac:dyDescent="0.3">
+      <c r="A56" s="22"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="35" t="s">
         <v>310</v>
       </c>
-      <c r="D52" s="35" t="s">
+      <c r="D56" s="35" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="22" t="s">
+    <row r="57" spans="1:4" ht="144" x14ac:dyDescent="0.3">
+      <c r="A57" s="22"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="35" t="s">
+        <v>302</v>
+      </c>
+      <c r="D57" s="21" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A58" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B53" s="17" t="s">
+      <c r="B58" s="17" t="s">
         <v>311</v>
       </c>
-      <c r="C53" s="35" t="s">
+      <c r="C58" s="35" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="144" x14ac:dyDescent="0.3">
-      <c r="C54" s="35" t="s">
-        <v>302</v>
-      </c>
-      <c r="D54" s="21" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="22" t="s">
+    <row r="59" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="C59" s="43" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B55" s="22" t="s">
+      <c r="B60" s="22" t="s">
         <v>190</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A47">
+  <conditionalFormatting sqref="A51">
     <cfRule type="duplicateValues" dxfId="3" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A27">
+  <conditionalFormatting sqref="A31">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A33">
+  <conditionalFormatting sqref="A37">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A55">
+  <conditionalFormatting sqref="A60">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="C21" r:id="rId1" xr:uid="{7A7102A8-672B-4BFA-9510-5628693AD70A}"/>
-    <hyperlink ref="C22" r:id="rId2" xr:uid="{5065060F-D999-41D2-A82D-C216F28E51A6}"/>
+    <hyperlink ref="C25" r:id="rId1" xr:uid="{7A7102A8-672B-4BFA-9510-5628693AD70A}"/>
+    <hyperlink ref="C26" r:id="rId2" xr:uid="{5065060F-D999-41D2-A82D-C216F28E51A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
   <drawing r:id="rId4"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F7C9A0E-4B49-46C5-A634-51A4C15E80AC}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:U90"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="39.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="21" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="76.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="21" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="6" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="6" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="21" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="21" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="21" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="7" customWidth="1"/>
+    <col min="21" max="21" width="67.77734375" style="21" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="8.77734375" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" s="8"/>
+      <c r="B2" s="51" t="s">
+        <v>429</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" s="11"/>
+      <c r="C3" s="15"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" s="11"/>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6" s="13"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" s="8"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="U9" s="4"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C11" s="43" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B12" s="22" t="s">
+        <v>367</v>
+      </c>
+      <c r="C12" s="49" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="C13" s="43" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="C14" s="43" t="s">
+        <v>405</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="C15" s="43" t="s">
+        <v>410</v>
+      </c>
+      <c r="D15" s="43" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="C16" s="43" t="s">
+        <v>414</v>
+      </c>
+      <c r="D16" s="43" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="52" t="s">
+        <v>435</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="C17" s="43" t="s">
+        <v>417</v>
+      </c>
+      <c r="D17" s="43" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="50" t="s">
+        <v>433</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="C18" s="43" t="s">
+        <v>419</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="50" t="s">
+        <v>433</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="C19" s="49" t="s">
+        <v>432</v>
+      </c>
+      <c r="D19" s="49" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="50" t="s">
+        <v>434</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="C20" s="43" t="s">
+        <v>421</v>
+      </c>
+      <c r="D20" s="43" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B21" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="C21" s="49" t="s">
+        <v>428</v>
+      </c>
+      <c r="D21" s="49" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="1"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B23" s="1"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B24" s="1"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B25" s="1"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B26" s="1"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="43"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B27" s="1"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B28" s="1"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B29" s="1"/>
+      <c r="C29" s="43"/>
+      <c r="D29" s="43"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B30" s="1"/>
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B31" s="1"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="43"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B32" s="1"/>
+      <c r="C32" s="43"/>
+      <c r="D32" s="43"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B33" s="1"/>
+      <c r="C33" s="43"/>
+      <c r="D33" s="43"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B34" s="1"/>
+      <c r="C34" s="43"/>
+      <c r="D34" s="31"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B35" s="1"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="31"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B36" s="1"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="31"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B37" s="1"/>
+      <c r="C37" s="43"/>
+      <c r="D37" s="31"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B38" s="1"/>
+      <c r="C38" s="43"/>
+      <c r="D38" s="31"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="11" t="s">
+        <v>385</v>
+      </c>
+      <c r="B39" s="1"/>
+      <c r="C39" s="43"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B40" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="C40" s="44" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B41" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C41" s="44" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="8" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B43" s="21" t="s">
+        <v>322</v>
+      </c>
+      <c r="C43" s="44" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B44" s="21" t="s">
+        <v>324</v>
+      </c>
+      <c r="C44" s="44" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="13" t="s">
+        <v>386</v>
+      </c>
+      <c r="C45" s="44"/>
+    </row>
+    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B46" s="21" t="s">
+        <v>326</v>
+      </c>
+      <c r="C46" s="44" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="B47" s="21" t="s">
+        <v>328</v>
+      </c>
+      <c r="C47" s="44"/>
+    </row>
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="44"/>
+      <c r="B48" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="C48" s="44" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B49" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="C49" s="44" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="C50" s="44"/>
+    </row>
+    <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B51" s="43" t="s">
+        <v>394</v>
+      </c>
+      <c r="C51" s="44" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A52" s="21" t="s">
+        <v>333</v>
+      </c>
+      <c r="B52" s="43" t="s">
+        <v>392</v>
+      </c>
+      <c r="C52" s="44" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A53" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="B53" s="43" t="s">
+        <v>391</v>
+      </c>
+      <c r="C53" s="44" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="C54" s="44"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B55" s="21" t="s">
+        <v>398</v>
+      </c>
+      <c r="C55" s="44" t="s">
+        <v>400</v>
+      </c>
+      <c r="D55" s="47" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B56" s="21" t="s">
+        <v>401</v>
+      </c>
+      <c r="C56" s="44" t="s">
+        <v>403</v>
+      </c>
+      <c r="D56" s="47" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="C57" s="44"/>
+    </row>
+    <row r="58" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A58" s="52"/>
+      <c r="B58" s="21" t="s">
+        <v>437</v>
+      </c>
+      <c r="C58" s="52" t="s">
+        <v>439</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B59" s="43" t="s">
+        <v>345</v>
+      </c>
+      <c r="C59" s="44" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B60" s="43" t="s">
+        <v>348</v>
+      </c>
+      <c r="C60" s="44" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B61" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="C61" s="44" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="43" t="s">
+        <v>341</v>
+      </c>
+      <c r="B62" s="45" t="s">
+        <v>346</v>
+      </c>
+      <c r="C62" s="44" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A63" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="B63" s="43" t="s">
+        <v>347</v>
+      </c>
+      <c r="C63" s="44" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+    </row>
+    <row r="65" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B65" s="43" t="s">
+        <v>358</v>
+      </c>
+      <c r="C65" s="44" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="144" x14ac:dyDescent="0.3">
+      <c r="B66" s="43" t="s">
+        <v>354</v>
+      </c>
+      <c r="C66" s="43" t="s">
+        <v>352</v>
+      </c>
+      <c r="D66" s="43" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="8" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="B68" s="17" t="s">
+        <v>360</v>
+      </c>
+      <c r="C68" s="44" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A69" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="B69" s="1"/>
+      <c r="C69" s="43"/>
+    </row>
+    <row r="70" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B70" s="21" t="s">
+        <v>366</v>
+      </c>
+      <c r="C70" s="44" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A71" s="46" t="s">
+        <v>369</v>
+      </c>
+      <c r="C71" s="44"/>
+    </row>
+    <row r="72" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B72" s="21" t="s">
+        <v>371</v>
+      </c>
+      <c r="C72" s="44" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A73" s="46" t="s">
+        <v>372</v>
+      </c>
+      <c r="C73" s="44"/>
+    </row>
+    <row r="74" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A74" s="21"/>
+      <c r="B74" s="21" t="s">
+        <v>379</v>
+      </c>
+      <c r="C74" s="44" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" s="21"/>
+      <c r="B75" s="48" t="s">
+        <v>378</v>
+      </c>
+      <c r="C75" s="44" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" s="21"/>
+      <c r="B76" s="21" t="s">
+        <v>375</v>
+      </c>
+      <c r="C76" s="44" t="s">
+        <v>376</v>
+      </c>
+      <c r="D76" s="47" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A77" s="21"/>
+      <c r="B77" s="21" t="s">
+        <v>381</v>
+      </c>
+      <c r="C77" s="44" t="s">
+        <v>380</v>
+      </c>
+      <c r="D77" s="44"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="46" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B79" s="21" t="s">
+        <v>365</v>
+      </c>
+      <c r="C79" s="44" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="13" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="81" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B81" s="21" t="s">
+        <v>384</v>
+      </c>
+      <c r="C81" s="44" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="85" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C85" s="43"/>
+    </row>
+    <row r="86" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C86" s="43"/>
+    </row>
+    <row r="88" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C88" s="43"/>
+    </row>
+    <row r="89" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C89" s="43"/>
+    </row>
+    <row r="90" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C90" s="43"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B99A4771-6185-4CF7-A0BE-E883D73AA38E}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:U13"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="39.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="50.5546875" style="21" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="76.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="21" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="6" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="6" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="21" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="21" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="21" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="7" customWidth="1"/>
+    <col min="21" max="21" width="67.77734375" style="21" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="8.77734375" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" s="8"/>
+      <c r="B2" s="51" t="s">
+        <v>429</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" s="11"/>
+      <c r="C3" s="15"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" s="11"/>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6" s="13"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" s="8"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="U9" s="4"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B11" s="52" t="s">
+        <v>440</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>446</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B12" s="21" t="s">
+        <v>444</v>
+      </c>
+      <c r="C12" s="49" t="s">
+        <v>445</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B13" s="21" t="s">
+        <v>448</v>
+      </c>
+      <c r="C13" s="49" t="s">
+        <v>449</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
save 24 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_26_Cursor.xlsx
+++ b/4 четверть_26_Cursor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36A76F0-AFC0-4E0A-A45C-5E9FA08AEE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADC6A08-B91E-433D-B90F-AF727D4BC2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-13875" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Учебные матриалы" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="476">
   <si>
     <t>Настройки Cursor</t>
   </si>
@@ -4244,17 +4244,38 @@
   <si>
     <t>Изучить</t>
   </si>
+  <si>
+    <t>open edit (command K) замени на ctrl + m
+замени все ctrl + m ... на ctrl + k ... в keybindings cursor</t>
+  </si>
+  <si>
+    <t>Перенос настроек Vscode в Cursor</t>
+  </si>
+  <si>
+    <t>Перенеси все extensions из vscode в cursor</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="31" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4570,9 +4591,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -4580,13 +4601,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4596,7 +4617,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4609,62 +4630,80 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -4673,88 +4712,73 @@
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="29" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4831,13 +4855,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>414130</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>61788</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>2113177</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>1200835</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -8056,7 +8080,7 @@
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:U54"/>
+  <dimension ref="A2:U58"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" style="1" customWidth="1"/>
@@ -8125,390 +8149,417 @@
       <c r="A8" s="21"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="4"/>
-      <c r="S9" s="4"/>
-      <c r="U9" s="4"/>
-    </row>
-    <row r="10" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" s="21" customFormat="1" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="35" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>354</v>
-      </c>
-      <c r="C12" s="35"/>
-    </row>
-    <row r="13" spans="1:21" s="21" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="C13" s="43" t="s">
-        <v>355</v>
-      </c>
+      <c r="A9" s="13" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" s="21"/>
+      <c r="B10" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="65" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="21"/>
+      <c r="B11" s="21" t="s">
+        <v>475</v>
+      </c>
+      <c r="C11" s="65" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12" s="21"/>
+      <c r="C12" s="65"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4"/>
+      <c r="U13" s="4"/>
     </row>
     <row r="14" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" s="21" customFormat="1" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="35" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="C16" s="35"/>
+    </row>
+    <row r="17" spans="1:4" s="21" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C17" s="43" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="21" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
         <v>285</v>
       </c>
-      <c r="C14" s="43"/>
-    </row>
-    <row r="15" spans="1:21" s="21" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="21" t="s">
+      <c r="C18" s="43"/>
+    </row>
+    <row r="19" spans="1:4" s="21" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="49" t="s">
+      <c r="C19" s="49" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="38"/>
-    </row>
-    <row r="17" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="35" t="s">
+      <c r="B20" s="36"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="38"/>
+    </row>
+    <row r="21" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="35" t="s">
         <v>274</v>
       </c>
-      <c r="B17" s="21" t="s">
+      <c r="B21" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="C17" s="42" t="s">
+      <c r="C21" s="42" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="21" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="21" t="s">
         <v>269</v>
       </c>
-      <c r="C18" s="42" t="s">
+      <c r="C22" s="42" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="64.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="21" t="s">
+    <row r="23" spans="1:4" ht="64.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="21" t="s">
         <v>271</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C23" s="35" t="s">
         <v>278</v>
       </c>
-      <c r="D19" s="35" t="s">
+      <c r="D23" s="35" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="35" t="s">
+    <row r="24" spans="1:4" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="35" t="s">
         <v>281</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D24" s="21" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B21" s="21" t="s">
+    <row r="25" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B25" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C25" s="35" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="35" t="s">
+    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="35" t="s">
         <v>275</v>
       </c>
-      <c r="B23" s="21" t="s">
+      <c r="B27" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C27" s="41" t="s">
         <v>312</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B24" s="21" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B28" s="21" t="s">
         <v>269</v>
       </c>
-      <c r="C24" s="41" t="s">
+      <c r="C28" s="41" t="s">
         <v>313</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B25" s="39" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B29" s="39" t="s">
         <v>291</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C29" s="31" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C26" s="16" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C30" s="16" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="13" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="13" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C28" s="41" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C32" s="41" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="17" t="s">
+    <row r="33" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="B29" s="21" t="s">
+      <c r="B33" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="C29" s="35"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="22" t="s">
+      <c r="C33" s="35"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B34" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="C30" s="35"/>
-    </row>
-    <row r="31" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="22" t="s">
+      <c r="C34" s="35"/>
+    </row>
+    <row r="35" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B31" s="35" t="s">
+      <c r="B35" s="35" t="s">
         <v>252</v>
       </c>
-      <c r="C31" s="35"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="39" t="s">
+      <c r="C35" s="35"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B36" s="39" t="s">
         <v>292</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="C36" s="15" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="8" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="17" t="s">
+    <row r="38" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B38" s="29" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="17" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B39" s="17" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="22" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B40" s="17" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="22" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B37" s="35" t="s">
+      <c r="B41" s="35" t="s">
         <v>294</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B38" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B39" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B40" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B41" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B42" s="34" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B43" s="40" t="s">
-        <v>67</v>
+      <c r="B43" s="24" t="s">
+        <v>59</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B44" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B45" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B46" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B47" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B48" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B45" s="24" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B49" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C49" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B46" s="21" t="s">
+    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B50" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C50" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="8" t="s">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="8" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A48" s="17" t="s">
+    <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="B48" s="29" t="s">
+      <c r="B52" s="29" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="17" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="17" t="s">
         <v>287</v>
       </c>
-      <c r="B49" s="21" t="s">
+      <c r="B53" s="21" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="22" t="s">
+    <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="B50" s="35" t="s">
+      <c r="B54" s="35" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="22" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B51" s="21" t="s">
+      <c r="B55" s="21" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="8" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="8" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="17" t="s">
+    <row r="57" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="B53" s="29" t="s">
+      <c r="B57" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="C53" s="57" t="s">
+      <c r="C57" s="57" t="s">
         <v>455</v>
       </c>
-      <c r="D53" s="1" t="s">
+      <c r="D57" s="1" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="22" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="B54" s="22" t="s">
+      <c r="B58" s="22" t="s">
         <v>190</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A51">
+  <conditionalFormatting sqref="A55">
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A31">
+  <conditionalFormatting sqref="A35">
     <cfRule type="duplicateValues" dxfId="3" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A37">
+  <conditionalFormatting sqref="A41">
     <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A54">
+  <conditionalFormatting sqref="A58">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="C25" r:id="rId1" xr:uid="{7A7102A8-672B-4BFA-9510-5628693AD70A}"/>
-    <hyperlink ref="C26" r:id="rId2" xr:uid="{5065060F-D999-41D2-A82D-C216F28E51A6}"/>
+    <hyperlink ref="C29" r:id="rId1" xr:uid="{7A7102A8-672B-4BFA-9510-5628693AD70A}"/>
+    <hyperlink ref="C30" r:id="rId2" xr:uid="{5065060F-D999-41D2-A82D-C216F28E51A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
@@ -9012,7 +9063,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="B12" s="22" t="s">
         <v>366</v>
       </c>

</xml_diff>

<commit_message>
save 28 07 2026
</commit_message>
<xml_diff>
--- a/4 четверть_26_Cursor.xlsx
+++ b/4 четверть_26_Cursor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADC6A08-B91E-433D-B90F-AF727D4BC2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10615DCF-9B00-4DCB-B3C4-E4639B0C5A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Учебные матриалы" sheetId="7" r:id="rId1"/>
@@ -4262,12 +4262,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4591,7 +4599,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -4601,13 +4609,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4617,7 +4625,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4630,62 +4638,80 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="25" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -4694,90 +4720,72 @@
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="30" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="29" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
save 21 08 2026
</commit_message>
<xml_diff>
--- a/4 четверть_26_Cursor.xlsx
+++ b/4 четверть_26_Cursor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7396809-315D-4C26-B886-5F25DF355782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84384690-457C-490E-A099-C19EAFE6C716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="1104" windowWidth="23016" windowHeight="11136" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Учебные матриалы" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="483">
   <si>
     <t>Настройки Cursor</t>
   </si>
@@ -1511,35 +1511,6 @@
 4. Answer using the fetched docs</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Попросить создать </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>rule</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">:
-</t>
-    </r>
-  </si>
-  <si>
     <t>Plugins</t>
   </si>
   <si>
@@ -3013,69 +2984,7 @@
     <t>Создание документации изменений для внешних пользователей</t>
   </si>
   <si>
-    <t>Before starting:
-- Run `git fetch origin main` to get latest changes
-- Check `git status` to understand current state
-- Verify you're on the correct branch
-During rebase:
-- Resolve conflicts one file at a time
-- After each file, run `grep -r "&lt;&lt;&lt;&lt;&lt;&lt;&lt; HEAD" . || echo "No conflicts"` to verify
-- For package-lock.json/yarn.lock: accept main version and run `npm install`
-- For binary files: escalate immediately (don't attempt to resolve)
-- For migrations: escalate if uncertain about semantics
-After rebase:
-- Run `git status` to verify rebase is complete
-- Run `npm test` to verify tests pass
-- If tests fail, check if it's due to your resolution or pre-existing issue
-- If due to your resolution, fix and re-test
-- If pre-existing, adapt your code to work with main changes
-Escape hatch:
-- If more than 5 conflicts or complex semantic conflicts, escalate instead of continuing
-- Use `git rebase --abort` only if rebase is completely broken</t>
-  </si>
-  <si>
     <t>Git</t>
-  </si>
-  <si>
-    <r>
-      <t>Разрешение rebase conflict 
-с т</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">екущей ветки </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-к ветке </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>main</t>
-    </r>
   </si>
   <si>
     <t>1 Создание документации изменений для внешних пользователей
@@ -4266,17 +4175,199 @@
   <si>
     <t>изучи @Browser https://www.sqlstyle.guide/ru/  и /create-skill  который бы форматировал sql запросы, не изменяя их, но корректируя табуляцию и правописание</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Попросить создать </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>rule</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Тогда даже без @Docs агент получает жёсткий контекст из правил + индекса кода.</t>
+    </r>
+  </si>
+  <si>
+    <t>Before starting:
+- Run 'git pull' to have the latest version of the project
+- Check `git status` to understand current state
+During revert:
+- Resolve conflicts one file at a time
+- After each file, run `grep -r "&lt;&lt;&lt;&lt;&lt;&lt;&lt; HEAD" . || echo "No conflicts"` to verify
+- For package-lock.json/yarn.lock: accept main version and run `npm install`
+- For binary files: escalate immediately (don't attempt to resolve)
+- For migrations: escalate if uncertain about semantics
+After revert:
+- Run `git status` to verify rebase is complete
+- Run `npm test` to verify tests pass
+- If tests fail, check if it's due to your resolution or pre-existing issue
+- If due to your resolution, fix and re-test
+- If pre-existing, adapt your code to work with main changes
+Escape hatch:
+- If more than 5 conflicts or complex semantic conflicts, escalate instead of continuing
+- Use `git revert --abort` only if revert is completely broken</t>
+  </si>
+  <si>
+    <r>
+      <t>Разрешение revert conflict 
+в т</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>екущей ветке</t>
+    </r>
+  </si>
+  <si>
+    <t>Before starting:
+- Run 'git pull' to have the latest version of the project
+- Check `git status` to understand current state
+During merge:
+- Resolve conflicts one file at a time
+- After each file, run `grep -r "&lt;&lt;&lt;&lt;&lt;&lt;&lt; HEAD" . || echo "No conflicts"` to verify
+- For package-lock.json/yarn.lock: accept main version and run `npm install`
+- For binary files: escalate immediately (don't attempt to resolve)
+- For migrations: escalate if uncertain about semantics
+After merge:
+- Run `git status` to verify rebase is complete
+- Run `npm test` to verify tests pass
+- If tests fail, check if it's due to your resolution or pre-existing issue
+- If due to your resolution, fix and re-test
+- If pre-existing, adapt your code to work with main changes
+Escape hatch:
+- If more than 5 conflicts or complex semantic conflicts, escalate instead of continuing
+- Use `git merge --abort` only if merge is completely broken</t>
+  </si>
+  <si>
+    <r>
+      <t>Разрешение merge conflict 
+текущая</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ветка &lt;- merge ветка</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Разрешение rebase conflict 
+т</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">екущая ветка </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">к rebase ветке </t>
+    </r>
+  </si>
+  <si>
+    <t>Before starting:
+- Run `git pull` of the branch to which rebase will be
+- Return to the target branch to be rebased
+- Check `git status` to understand current state
+- Verify you're on the correct branch
+During rebase:
+- Resolve conflicts one file at a time
+- After each file, run `grep -r "&lt;&lt;&lt;&lt;&lt;&lt;&lt; HEAD" . || echo "No conflicts"` to verify
+- For package-lock.json/yarn.lock: accept main version and run `npm install`
+- For binary files: escalate immediately (don't attempt to resolve)
+- For migrations: escalate if uncertain about semantics
+After rebase:
+- Run `git status` to verify rebase is complete
+- Run `npm test` to verify tests pass
+- If tests fail, check if it's due to your resolution or pre-existing issue
+- If due to your resolution, fix and re-test
+- If pre-existing, adapt your code to work with main changes
+Escape hatch:
+- If more than 5 conflicts or complex semantic conflicts, escalate instead of continuing
+- Use `git rebase --abort` only if rebase is completely broken</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="34" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4616,9 +4707,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -4626,13 +4717,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4642,7 +4733,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4655,90 +4746,120 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -4746,69 +4867,42 @@
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="33" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="33" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="31" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5259,13 +5353,13 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="60" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="C7" s="59" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
   </sheetData>
@@ -7124,7 +7218,7 @@
         <v>186</v>
       </c>
       <c r="D65" s="28" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F65" s="1"/>
       <c r="G65" s="21"/>
@@ -7452,7 +7546,7 @@
     <row r="79" spans="1:21" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A79" s="21"/>
       <c r="B79" s="21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C79" s="21"/>
       <c r="D79" s="21"/>
@@ -7473,7 +7567,7 @@
     </row>
     <row r="80" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B80" s="21"/>
       <c r="C80" s="3"/>
@@ -7926,10 +8020,10 @@
     <row r="99" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A99" s="21"/>
       <c r="B99" s="21" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="C99" s="58" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="D99" s="1"/>
       <c r="F99" s="1"/>
@@ -8181,7 +8275,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
@@ -8190,16 +8284,16 @@
         <v>53</v>
       </c>
       <c r="C10" s="65" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="21"/>
       <c r="B11" s="21" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="C11" s="65" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
@@ -8227,28 +8321,28 @@
     </row>
     <row r="14" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:21" s="21" customFormat="1" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="35" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="16" spans="1:21" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C16" s="35"/>
     </row>
     <row r="17" spans="1:4" s="21" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="C17" s="43" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="18" spans="1:4" s="21" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C18" s="43"/>
     </row>
@@ -8256,8 +8350,8 @@
       <c r="B19" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="49" t="s">
-        <v>442</v>
+      <c r="C19" s="68" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -8276,7 +8370,7 @@
         <v>268</v>
       </c>
       <c r="C21" s="42" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -8298,87 +8392,87 @@
         <v>279</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C24" s="35" t="s">
-        <v>281</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B25" s="21" t="s">
+    <row r="24" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B24" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C25" s="35" t="s">
+      <c r="C24" s="68" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="13" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="35" t="s">
+    <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="35" t="s">
         <v>275</v>
       </c>
+      <c r="B26" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="C26" s="41" t="s">
+        <v>311</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B27" s="21" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C27" s="41" t="s">
         <v>312</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="21" t="s">
-        <v>269</v>
-      </c>
-      <c r="C28" s="41" t="s">
-        <v>313</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>277</v>
+      <c r="B28" s="39" t="s">
+        <v>290</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B29" s="39" t="s">
-        <v>291</v>
-      </c>
-      <c r="C29" s="31" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C30" s="16" t="s">
+      <c r="C29" s="16" t="s">
         <v>135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="331.2" x14ac:dyDescent="0.3">
+      <c r="B30" s="68" t="s">
+        <v>476</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C32" s="41" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C33" s="35"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B34" s="17" t="s">
         <v>243</v>
@@ -8387,7 +8481,7 @@
     </row>
     <row r="35" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B35" s="35" t="s">
         <v>252</v>
@@ -8396,7 +8490,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B36" s="39" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>238</v>
@@ -8404,12 +8498,12 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="17" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B38" s="29" t="s">
         <v>48</v>
@@ -8417,15 +8511,15 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B40" s="17" t="s">
         <v>78</v>
@@ -8433,10 +8527,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B41" s="35" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -8518,7 +8612,7 @@
     </row>
     <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52" s="17" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B52" s="29" t="s">
         <v>152</v>
@@ -8526,23 +8620,23 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B53" s="21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="22" t="s">
+        <v>287</v>
+      </c>
+      <c r="B54" s="35" t="s">
         <v>288</v>
-      </c>
-      <c r="B54" s="35" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B55" s="21" t="s">
         <v>171</v>
@@ -8550,26 +8644,26 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A57" s="17" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B57" s="29" t="s">
+        <v>302</v>
+      </c>
+      <c r="C57" s="57" t="s">
+        <v>452</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="C57" s="57" t="s">
-        <v>455</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B58" s="22" t="s">
         <v>190</v>
@@ -8589,8 +8683,8 @@
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="C29" r:id="rId1" xr:uid="{7A7102A8-672B-4BFA-9510-5628693AD70A}"/>
-    <hyperlink ref="C30" r:id="rId2" xr:uid="{5065060F-D999-41D2-A82D-C216F28E51A6}"/>
+    <hyperlink ref="C28" r:id="rId1" xr:uid="{7A7102A8-672B-4BFA-9510-5628693AD70A}"/>
+    <hyperlink ref="C29" r:id="rId2" xr:uid="{5065060F-D999-41D2-A82D-C216F28E51A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
@@ -8663,7 +8757,7 @@
       <c r="A4" s="21"/>
       <c r="B4" s="21"/>
       <c r="C4" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D4" s="1"/>
       <c r="F4" s="1"/>
@@ -8683,7 +8777,7 @@
     </row>
     <row r="5" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -8705,14 +8799,14 @@
     </row>
     <row r="6" spans="1:21" s="6" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="29" t="s">
+        <v>302</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="21"/>
@@ -8731,11 +8825,11 @@
     </row>
     <row r="7" spans="1:21" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B7" s="21"/>
       <c r="C7" s="57" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="D7" s="1"/>
       <c r="F7" s="1"/>
@@ -8755,7 +8849,7 @@
     </row>
     <row r="8" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="35"/>
@@ -8777,16 +8871,16 @@
     </row>
     <row r="9" spans="1:21" s="6" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="B9" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="C9" s="35" t="s">
         <v>305</v>
       </c>
-      <c r="C9" s="35" t="s">
-        <v>306</v>
-      </c>
       <c r="D9" s="35" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="21"/>
@@ -8805,14 +8899,14 @@
     </row>
     <row r="10" spans="1:21" s="6" customFormat="1" ht="216" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="35" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D10" s="57" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="21"/>
@@ -8831,14 +8925,14 @@
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="35" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="21"/>
@@ -8857,7 +8951,7 @@
     </row>
     <row r="12" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="35"/>
@@ -8879,13 +8973,13 @@
     </row>
     <row r="13" spans="1:21" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C13" s="35" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D13" s="1"/>
       <c r="F13" s="1"/>
@@ -8907,7 +9001,7 @@
       <c r="A14" s="1"/>
       <c r="B14" s="21"/>
       <c r="C14" s="43" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D14" s="1"/>
       <c r="F14" s="1"/>
@@ -8927,7 +9021,7 @@
     </row>
     <row r="15" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B15" s="22" t="s">
         <v>190</v>
@@ -8951,34 +9045,34 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="C18" s="57" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="C19" s="57" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
   </sheetData>
@@ -8996,7 +9090,7 @@
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:U77"/>
+  <dimension ref="A2:U79"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" style="1" customWidth="1"/>
@@ -9032,10 +9126,10 @@
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="51" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
@@ -9048,12 +9142,12 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="62" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" s="63" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
@@ -9083,156 +9177,156 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="B12" s="22" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C12" s="61" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C13" s="57" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B14" s="21" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="C16" s="53" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C17" s="43"/>
       <c r="D17" s="43" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="C18" s="43" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D18" s="43" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="52" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="C19" s="43" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="D19" s="56" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="50" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="C20" s="43" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D20" s="53" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="50" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C21" s="49" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="D21" s="49" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A22" s="50" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="C22" s="57" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="D22" s="53" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="C23" s="49" t="s">
         <v>417</v>
       </c>
-      <c r="C23" s="49" t="s">
-        <v>420</v>
-      </c>
       <c r="D23" s="49" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="49"/>
@@ -9240,177 +9334,177 @@
     </row>
     <row r="25" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="C25" s="67" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="D25" s="49"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="62" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="43"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="C27" s="64" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B28" s="1" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C28" s="44" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
       <c r="B30" s="21" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C30" s="66" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
       <c r="B31" s="21" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C31" s="66" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="13" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C32" s="44"/>
     </row>
     <row r="33" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B33" s="21" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C33" s="44" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="63" t="s">
+        <v>325</v>
+      </c>
+      <c r="B34" s="21" t="s">
         <v>326</v>
-      </c>
-      <c r="B34" s="21" t="s">
-        <v>327</v>
       </c>
       <c r="C34" s="44"/>
     </row>
     <row r="35" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A35" s="44"/>
       <c r="B35" s="21" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B36" s="21" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C36" s="44" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C37" s="44"/>
     </row>
     <row r="38" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B38" s="53" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="C38" s="54" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A39" s="21" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B39" s="53" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="C39" s="54" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A40" s="21" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B40" s="43" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C40" s="44" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C41" s="44"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B42" s="21" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="C42" s="44" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="D42" s="47" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
       <c r="B43" s="21" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="C43" s="53" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="D43" s="55" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C44" s="44"/>
     </row>
     <row r="45" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="52"/>
       <c r="B45" s="21" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C45" s="52" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
@@ -9418,213 +9512,229 @@
         <v>53</v>
       </c>
       <c r="B46" s="43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C46" s="44" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B47" s="43" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C47" s="44" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C48" s="44" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A49" s="43" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B49" s="45" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C49" s="44" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A50" s="43" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B50" s="43" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C50" s="44" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
     </row>
     <row r="52" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B52" s="43" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C52" s="44" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="B53" s="43" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C53" s="43" t="s">
+        <v>350</v>
+      </c>
+      <c r="D53" s="43" t="s">
         <v>351</v>
-      </c>
-      <c r="D53" s="43" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B55" s="17" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C55" s="44" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="46" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B56" s="1"/>
       <c r="C56" s="43"/>
     </row>
     <row r="57" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B57" s="21" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C57" s="44" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" s="46" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C58" s="44"/>
     </row>
     <row r="59" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B59" s="21" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C59" s="44" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A60" s="46" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C60" s="44"/>
     </row>
     <row r="61" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A61" s="21"/>
       <c r="B61" s="21" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C61" s="44" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="21"/>
       <c r="B62" s="48" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C62" s="44" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="21"/>
       <c r="B63" s="21" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C63" s="44" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="D63" s="47" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A64" s="21"/>
       <c r="B64" s="21" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C64" s="44" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="D64" s="44"/>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="46" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B66" s="21" t="s">
-        <v>364</v>
+        <v>481</v>
       </c>
       <c r="C66" s="44" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="13" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B67" s="21" t="s">
+        <v>478</v>
+      </c>
+      <c r="C67" s="44" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B68" s="21" t="s">
-        <v>382</v>
+        <v>480</v>
       </c>
       <c r="C68" s="44" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C72" s="43"/>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C73" s="43"/>
+        <v>479</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="13" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B70" s="21" t="s">
+        <v>379</v>
+      </c>
+      <c r="C70" s="44" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C74" s="43"/>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C75" s="43"/>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C76" s="43"/>
-    </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C77" s="43"/>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C78" s="43"/>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C79" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9673,10 +9783,10 @@
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="51" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
@@ -9720,43 +9830,43 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C11" s="49" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B12" s="21" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="C12" s="49" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="C13" s="49" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
save 26 08 2024
</commit_message>
<xml_diff>
--- a/4 четверть_26_Cursor.xlsx
+++ b/4 четверть_26_Cursor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF78AB23-238F-4930-9AC9-3859116A9F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42BE39B-21BA-4608-B6AE-2DE9156E7AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-420" yWindow="-16155" windowWidth="18405" windowHeight="13470" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Учебные матриалы" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="506">
   <si>
     <t>Настройки Cursor</t>
   </si>
@@ -3174,9 +3174,6 @@
   </si>
   <si>
     <t xml:space="preserve">/using-superpowers - Я собираюсь переписать проект с graphql на rest. Пройди по этим шагам: Шаг 1: сформулируй, что именно я решаю. Шаг 2: назови три альтернативных подхода. Шаг 3: для каждого — плюсы, минусы, когда подходит. Шаг 4: дай рекомендацию с обоснованием. Не пропускай шаги, не объединяй их. </t>
-  </si>
-  <si>
-    <t>Запрос 1</t>
   </si>
   <si>
     <t>Запрос 2</t>
@@ -4355,17 +4352,241 @@
 Причина: у компании Innovatika Primorye нет пользователей. При сохранении по кнопке «Сохранить для всех пользователей и шаблон компании» backend всё равно запускал массовое обновление пользователей и формировал SQL с пустым условием IN (). Выполнение прерывалось до сохранения параметров самой компании, поэтому блокировка не применялась. Отдельная кнопка «Сохранить шаблон компании» этот маршрут обходила и работала.
 Исправление: при пустом списке пользователей пользовательская часть массового сохранения пропускается, после чего параметры компании, включая блокировку, сохраняются штатно. Добавлена регрессионная проверка.</t>
   </si>
+  <si>
+    <t>http://auth.linux.hwc.ldom</t>
+  </si>
+  <si>
+    <t>Code refactoring</t>
+  </si>
+  <si>
+    <t>Refactor this code to make it simpler, remove duplication and overengineering without changing functionality</t>
+  </si>
+  <si>
+    <t>Прямого встроенного аналога команды /simplify из Claude Code (которая запускает параллельных субагентов для очистки git diff от избыточности и оверинжиниринга) в виде одной кнопки или аналогичного слэш-кода в Cursor нет.</t>
+  </si>
+  <si>
+    <t>/create-skill Ниже будет план действий с вложенными изображениями. Принимай каждый пункт плана без обработки пока не получишь сообщения "составь свой план реализации на основе переданных пунктов"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Когда нет конкретного плана действий</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Запрос 1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Когда понятны конкретные действия</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, которые нужно сделать
+/deferred-plan-accumulation</t>
+    </r>
+  </si>
+  <si>
+    <t>Work summary</t>
+  </si>
+  <si>
+    <t>Что должен протестировать ручной тестировщик</t>
+  </si>
+  <si>
+    <t>`https://github.com/unlearndev/skills/tree/main/skills/qa-checklist</t>
+  </si>
+  <si>
+    <t>Code-review</t>
+  </si>
+  <si>
+    <t>`https://github.com/unlearndev/skills/blob/main/skills/judge-arch/SKILL.md</t>
+  </si>
+  <si>
+    <t>Если есть файл DECISIONS.md
+В файле должны быть указаны BEST Practices для построения арзитектуры проекта</t>
+  </si>
+  <si>
+    <t>Промпт 1 - CHANGEABILITY
+"Challenge this design for long-term changeability. What change does it make hardest?"
+Промпт 2 - COUPLING &amp; OWNERSHIP
+"Find the coupling and ownership problems in this change."
+Промпт 3 - SIMPLER
+"Propose a simpler structure that still meets the requirements. What would we lose?"</t>
+  </si>
+  <si>
+    <t>Make the critic a habit
+01 When the change is done, open a fresh session (not the one that wrote the code).
+02 Ask for problems, not approval. "Is this good?" gets you a compliment.
+03 Findings only: tell it not to write code. You decide what gets fixed.</t>
+  </si>
+  <si>
+    <t>/create-skill
+Запустить отдельного агента (новый чат) с другой моделью</t>
+  </si>
+  <si>
+    <t>Architecture Decision Records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Только для разработки в команде (не имеет смысла, если один разработчик на проекте)
+</t>
+  </si>
+  <si>
+    <t>Исполнение в строгом соответсвии с правилами кодинга</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Когда хочешь, чтобы </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ИИ выполнил работу строго в соответствии с определенным паттерном</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> проектирования</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Point at an existing module</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+"Structure this like app/Domain/Billing."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Point at a web resource</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+"Read https://stitcher.io/blog/laravel-beyond-crud and structure the new billing"
+"Match the module layout of github.com/spatie/laravel-medialibrary for our uploads rewrite."</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="41" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4729,9 +4950,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -4739,13 +4960,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4755,7 +4976,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4768,58 +4989,88 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="28" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -4829,19 +5080,25 @@
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -4850,47 +5107,31 @@
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="38" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="38" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -4898,22 +5139,11 @@
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="34" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -4930,8 +5160,14 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5040,6 +5276,99 @@
         <a:xfrm>
           <a:off x="3097695" y="1883962"/>
           <a:ext cx="1695237" cy="1142857"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>707874</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>459908</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3103383</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>1428486</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Рисунок 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2D797F9-6157-4A17-8846-AD904EEE54EC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3397286" y="10612437"/>
+          <a:ext cx="2399319" cy="972388"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>181198</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>52584</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3070030</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>1006393</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Рисунок 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C7B8DF7-E888-4E67-B3A7-6EE0A3CEFCEC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6333227" y="10205113"/>
+          <a:ext cx="2888832" cy="948094"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5380,14 +5709,14 @@
       <c r="U5" s="4"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A7" s="60" t="s">
-        <v>468</v>
+      <c r="A7" s="59" t="s">
+        <v>467</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>467</v>
-      </c>
-      <c r="C7" s="59" t="s">
         <v>466</v>
+      </c>
+      <c r="C7" s="58" t="s">
+        <v>465</v>
       </c>
     </row>
   </sheetData>
@@ -8026,7 +8355,7 @@
     <row r="98" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A98" s="21"/>
       <c r="B98" s="21"/>
-      <c r="C98" s="57" t="s">
+      <c r="C98" s="56" t="s">
         <v>74</v>
       </c>
       <c r="D98" s="1"/>
@@ -8048,10 +8377,10 @@
     <row r="99" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A99" s="21"/>
       <c r="B99" s="21" t="s">
+        <v>462</v>
+      </c>
+      <c r="C99" s="57" t="s">
         <v>463</v>
-      </c>
-      <c r="C99" s="58" t="s">
-        <v>464</v>
       </c>
       <c r="D99" s="1"/>
       <c r="F99" s="1"/>
@@ -8303,7 +8632,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
@@ -8311,22 +8640,22 @@
       <c r="B10" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="65" t="s">
-        <v>471</v>
+      <c r="C10" s="64" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="21"/>
       <c r="B11" s="21" t="s">
-        <v>472</v>
-      </c>
-      <c r="C11" s="65" t="s">
-        <v>469</v>
+        <v>471</v>
+      </c>
+      <c r="C11" s="64" t="s">
+        <v>468</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="21"/>
-      <c r="C12" s="65"/>
+      <c r="C12" s="64"/>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -8410,7 +8739,7 @@
       <c r="B22" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C22" s="68" t="s">
+      <c r="C22" s="67" t="s">
         <v>273</v>
       </c>
     </row>
@@ -8458,8 +8787,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="331.2" x14ac:dyDescent="0.3">
-      <c r="B28" s="68" t="s">
-        <v>476</v>
+      <c r="B28" s="67" t="s">
+        <v>475</v>
       </c>
       <c r="C28" s="21" t="s">
         <v>280</v>
@@ -8621,10 +8950,10 @@
     </row>
     <row r="49" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
       <c r="B49" s="21" t="s">
-        <v>484</v>
-      </c>
-      <c r="C49" s="70" t="s">
-        <v>439</v>
+        <v>483</v>
+      </c>
+      <c r="C49" s="69" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
@@ -8667,10 +8996,10 @@
     <row r="55" spans="1:4" ht="216" x14ac:dyDescent="0.3">
       <c r="A55" s="22"/>
       <c r="B55" s="21" t="s">
-        <v>483</v>
-      </c>
-      <c r="C55" s="70" t="s">
-        <v>485</v>
+        <v>482</v>
+      </c>
+      <c r="C55" s="69" t="s">
+        <v>484</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
@@ -8688,8 +9017,8 @@
       <c r="B58" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="C58" s="57" t="s">
-        <v>452</v>
+      <c r="C58" s="56" t="s">
+        <v>451</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>303</v>
@@ -8862,8 +9191,8 @@
         <v>286</v>
       </c>
       <c r="B7" s="21"/>
-      <c r="C7" s="57" t="s">
-        <v>447</v>
+      <c r="C7" s="56" t="s">
+        <v>446</v>
       </c>
       <c r="D7" s="1"/>
       <c r="F7" s="1"/>
@@ -8883,7 +9212,7 @@
     </row>
     <row r="8" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="35"/>
@@ -8905,7 +9234,7 @@
     </row>
     <row r="9" spans="1:21" s="6" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>304</v>
@@ -8933,13 +9262,13 @@
     </row>
     <row r="10" spans="1:21" s="6" customFormat="1" ht="216" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="35" t="s">
         <v>308</v>
       </c>
-      <c r="D10" s="57" t="s">
+      <c r="D10" s="56" t="s">
         <v>307</v>
       </c>
       <c r="F10" s="1"/>
@@ -8959,7 +9288,7 @@
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="35" t="s">
@@ -8985,7 +9314,7 @@
     </row>
     <row r="12" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="35"/>
@@ -9079,34 +9408,34 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="B17" s="57" t="s">
-        <v>454</v>
-      </c>
-      <c r="C17" s="57" t="s">
+        <v>458</v>
+      </c>
+      <c r="B17" s="56" t="s">
         <v>453</v>
+      </c>
+      <c r="C17" s="56" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="C18" s="57" t="s">
-        <v>455</v>
+        <v>457</v>
+      </c>
+      <c r="C18" s="56" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="C19" s="57" t="s">
         <v>456</v>
+      </c>
+      <c r="C19" s="56" t="s">
+        <v>455</v>
       </c>
     </row>
   </sheetData>
@@ -9124,7 +9453,7 @@
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:U79"/>
+  <dimension ref="A2:U94"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" style="1" customWidth="1"/>
@@ -9160,10 +9489,10 @@
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="51" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
@@ -9175,12 +9504,12 @@
       <c r="C4" s="15"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="61" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="62" t="s">
         <v>325</v>
       </c>
     </row>
@@ -9226,553 +9555,678 @@
       <c r="B12" s="22" t="s">
         <v>363</v>
       </c>
-      <c r="C12" s="61" t="s">
-        <v>460</v>
+      <c r="C12" s="60" t="s">
+        <v>459</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
-        <v>444</v>
-      </c>
-      <c r="C13" s="57" t="s">
-        <v>461</v>
+        <v>443</v>
+      </c>
+      <c r="C13" s="56" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B14" s="21" t="s">
-        <v>465</v>
-      </c>
-      <c r="C14" s="58" t="s">
         <v>464</v>
+      </c>
+      <c r="C14" s="57" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="C15" s="57" t="s">
         <v>442</v>
+      </c>
+      <c r="C15" s="56" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C16" s="53" t="s">
         <v>397</v>
       </c>
-      <c r="C16" s="53" t="s">
+      <c r="D16" s="21" t="s">
         <v>398</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C17" s="43"/>
       <c r="D17" s="43" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C18" s="43" t="s">
         <v>403</v>
       </c>
-      <c r="C18" s="43" t="s">
-        <v>404</v>
-      </c>
       <c r="D18" s="43" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="52" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="C19" s="43" t="s">
         <v>406</v>
       </c>
-      <c r="C19" s="43" t="s">
-        <v>407</v>
-      </c>
-      <c r="D19" s="56" t="s">
-        <v>405</v>
+      <c r="D19" s="55" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="50" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C20" s="43" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D20" s="53" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="50" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="C21" s="49" t="s">
         <v>420</v>
       </c>
-      <c r="C21" s="49" t="s">
-        <v>421</v>
-      </c>
       <c r="D21" s="49" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A22" s="50" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="C22" s="56" t="s">
+        <v>461</v>
+      </c>
+      <c r="D22" s="53" t="s">
         <v>411</v>
-      </c>
-      <c r="C22" s="57" t="s">
-        <v>462</v>
-      </c>
-      <c r="D22" s="53" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C23" s="49" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D23" s="49" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
-        <v>473</v>
-      </c>
       <c r="B24" s="1"/>
       <c r="C24" s="49"/>
       <c r="D24" s="49"/>
     </row>
-    <row r="25" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B25" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="C25" s="67" t="s">
-        <v>475</v>
-      </c>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B25" s="1"/>
+      <c r="C25" s="49"/>
       <c r="D25" s="49"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="62" t="s">
-        <v>380</v>
+      <c r="A26" s="8" t="s">
+        <v>501</v>
       </c>
       <c r="B26" s="1"/>
-      <c r="C26" s="43"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B27" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="C27" s="64" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="C28" s="44" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="B30" s="21" t="s">
-        <v>320</v>
-      </c>
-      <c r="C30" s="66" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="B31" s="21" t="s">
-        <v>322</v>
-      </c>
-      <c r="C31" s="66" t="s">
-        <v>321</v>
-      </c>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+    </row>
+    <row r="27" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B27" s="74" t="s">
+        <v>502</v>
+      </c>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+    </row>
+    <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="75" t="s">
+        <v>503</v>
+      </c>
+      <c r="B28" s="74"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+    </row>
+    <row r="29" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B29" s="74"/>
+      <c r="C29" s="74" t="s">
+        <v>505</v>
+      </c>
+      <c r="D29" s="49"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="61" t="s">
+        <v>492</v>
+      </c>
+      <c r="B30" s="1"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B31" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="C31" s="74" t="s">
+        <v>494</v>
+      </c>
+      <c r="D31" s="49"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="C32" s="44"/>
-    </row>
-    <row r="33" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="61" t="s">
+        <v>495</v>
+      </c>
+      <c r="B32" s="1"/>
+      <c r="C32" s="74"/>
+      <c r="D32" s="49"/>
+    </row>
+    <row r="33" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B33" s="21" t="s">
-        <v>324</v>
-      </c>
-      <c r="C33" s="44" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="63" t="s">
-        <v>325</v>
-      </c>
+        <v>500</v>
+      </c>
+      <c r="C33" s="74" t="s">
+        <v>498</v>
+      </c>
+      <c r="D33" s="74" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B34" s="21" t="s">
-        <v>326</v>
-      </c>
-      <c r="C34" s="44"/>
-    </row>
-    <row r="35" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="44"/>
-      <c r="B35" s="21" t="s">
-        <v>329</v>
-      </c>
-      <c r="C35" s="56" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B36" s="21" t="s">
-        <v>329</v>
-      </c>
-      <c r="C36" s="44" t="s">
-        <v>327</v>
-      </c>
+        <v>497</v>
+      </c>
+      <c r="C34" s="74" t="s">
+        <v>496</v>
+      </c>
+      <c r="D34" s="49"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>486</v>
+      </c>
+      <c r="B35" s="1"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="49"/>
+    </row>
+    <row r="36" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="B36" s="71" t="s">
+        <v>488</v>
+      </c>
+      <c r="C36" s="74" t="s">
+        <v>487</v>
+      </c>
+      <c r="D36" s="49"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
-        <v>387</v>
-      </c>
-      <c r="C37" s="44"/>
-    </row>
-    <row r="38" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B38" s="53" t="s">
-        <v>440</v>
-      </c>
-      <c r="C38" s="54" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A39" s="21" t="s">
-        <v>331</v>
-      </c>
-      <c r="B39" s="53" t="s">
-        <v>441</v>
-      </c>
-      <c r="C39" s="54" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A40" s="21" t="s">
-        <v>332</v>
-      </c>
-      <c r="B40" s="43" t="s">
-        <v>386</v>
-      </c>
-      <c r="C40" s="44" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="8" t="s">
-        <v>390</v>
-      </c>
-      <c r="C41" s="44"/>
+        <v>472</v>
+      </c>
+      <c r="B37" s="1"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="49"/>
+    </row>
+    <row r="38" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B38" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="C38" s="66" t="s">
+        <v>474</v>
+      </c>
+      <c r="D38" s="49"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="61" t="s">
+        <v>380</v>
+      </c>
+      <c r="B39" s="1"/>
+      <c r="C39" s="43"/>
+    </row>
+    <row r="40" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B40" s="72" t="s">
+        <v>491</v>
+      </c>
+      <c r="C40" s="72" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="106.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="74" t="s">
+        <v>504</v>
+      </c>
+      <c r="C41" s="74" t="s">
+        <v>505</v>
+      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B42" s="21" t="s">
-        <v>391</v>
-      </c>
-      <c r="C42" s="44" t="s">
-        <v>393</v>
-      </c>
-      <c r="D42" s="47" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="B43" s="21" t="s">
-        <v>394</v>
-      </c>
-      <c r="C43" s="53" t="s">
-        <v>396</v>
-      </c>
-      <c r="D43" s="55" t="s">
-        <v>395</v>
+      <c r="B42" s="73" t="s">
+        <v>490</v>
+      </c>
+      <c r="C42" s="63" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B43" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="C43" s="44" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="B45" s="21" t="s">
+        <v>320</v>
+      </c>
+      <c r="C45" s="70" t="s">
+        <v>318</v>
+      </c>
+      <c r="D45" s="31" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="B46" s="21" t="s">
+        <v>322</v>
+      </c>
+      <c r="C46" s="65" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="C47" s="44"/>
+    </row>
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B48" s="21" t="s">
+        <v>324</v>
+      </c>
+      <c r="C48" s="44" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="62" t="s">
+        <v>325</v>
+      </c>
+      <c r="B49" s="21" t="s">
+        <v>326</v>
+      </c>
+      <c r="C49" s="44"/>
+    </row>
+    <row r="50" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A50" s="44"/>
+      <c r="B50" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="C50" s="55" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B51" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="C51" s="44" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="C52" s="44"/>
+    </row>
+    <row r="53" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="B53" s="53" t="s">
+        <v>439</v>
+      </c>
+      <c r="C53" s="54" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A54" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="B54" s="53" t="s">
+        <v>440</v>
+      </c>
+      <c r="C54" s="54" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A55" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="B55" s="43" t="s">
+        <v>385</v>
+      </c>
+      <c r="C55" s="44" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="C56" s="44"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B57" s="21" t="s">
+        <v>390</v>
+      </c>
+      <c r="C57" s="44" t="s">
+        <v>392</v>
+      </c>
+      <c r="D57" s="47" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B58" s="21" t="s">
+        <v>393</v>
+      </c>
+      <c r="C58" s="44" t="s">
+        <v>395</v>
+      </c>
+      <c r="D58" s="47" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="C44" s="44"/>
-    </row>
-    <row r="45" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="52"/>
-      <c r="B45" s="21" t="s">
+      <c r="C59" s="44"/>
+    </row>
+    <row r="60" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A60" s="52"/>
+      <c r="B60" s="21" t="s">
+        <v>425</v>
+      </c>
+      <c r="C60" s="52" t="s">
+        <v>427</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="C45" s="52" t="s">
-        <v>428</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
+    </row>
+    <row r="61" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B46" s="43" t="s">
+      <c r="B61" s="43" t="s">
         <v>343</v>
       </c>
-      <c r="C46" s="44" t="s">
+      <c r="C61" s="44" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
+    <row r="62" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="B47" s="43" t="s">
+      <c r="B62" s="43" t="s">
         <v>346</v>
       </c>
-      <c r="C47" s="44" t="s">
+      <c r="C62" s="44" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+    <row r="63" spans="1:4" ht="259.2" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B63" s="17" t="s">
         <v>347</v>
       </c>
-      <c r="C48" s="44" t="s">
+      <c r="C63" s="44" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="43" t="s">
+    <row r="64" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A64" s="43" t="s">
         <v>339</v>
       </c>
-      <c r="B49" s="45" t="s">
+      <c r="B64" s="45" t="s">
         <v>344</v>
       </c>
-      <c r="C49" s="44" t="s">
+      <c r="C64" s="44" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A50" s="43" t="s">
+    <row r="65" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A65" s="43" t="s">
         <v>340</v>
       </c>
-      <c r="B50" s="43" t="s">
+      <c r="B65" s="43" t="s">
         <v>345</v>
       </c>
-      <c r="C50" s="44" t="s">
+      <c r="C65" s="44" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="8" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-    </row>
-    <row r="52" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B52" s="43" t="s">
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+    </row>
+    <row r="67" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B67" s="43" t="s">
         <v>356</v>
       </c>
-      <c r="C52" s="44" t="s">
+      <c r="C67" s="44" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="144" x14ac:dyDescent="0.3">
-      <c r="B53" s="43" t="s">
+    <row r="68" spans="1:4" ht="144" x14ac:dyDescent="0.3">
+      <c r="B68" s="43" t="s">
         <v>352</v>
       </c>
-      <c r="C53" s="43" t="s">
+      <c r="C68" s="43" t="s">
         <v>350</v>
       </c>
-      <c r="D53" s="43" t="s">
+      <c r="D68" s="43" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="8" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="8" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B55" s="17" t="s">
+    <row r="70" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="B70" s="17" t="s">
         <v>358</v>
       </c>
-      <c r="C55" s="44" t="s">
+      <c r="C70" s="44" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A56" s="46" t="s">
+    <row r="71" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A71" s="46" t="s">
         <v>360</v>
       </c>
-      <c r="B56" s="1"/>
-      <c r="C56" s="43"/>
-    </row>
-    <row r="57" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="21" t="s">
+      <c r="B71" s="1"/>
+      <c r="C71" s="43"/>
+    </row>
+    <row r="72" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B72" s="21" t="s">
         <v>362</v>
       </c>
-      <c r="C57" s="44" t="s">
+      <c r="C72" s="44" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A58" s="46" t="s">
+    <row r="73" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A73" s="46" t="s">
         <v>364</v>
       </c>
-      <c r="C58" s="44"/>
-    </row>
-    <row r="59" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B59" s="21" t="s">
+      <c r="C73" s="44"/>
+    </row>
+    <row r="74" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B74" s="21" t="s">
         <v>366</v>
       </c>
-      <c r="C59" s="44" t="s">
+      <c r="C74" s="44" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A60" s="46" t="s">
+    <row r="75" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A75" s="46" t="s">
         <v>367</v>
       </c>
-      <c r="C60" s="44"/>
-    </row>
-    <row r="61" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A61" s="21"/>
-      <c r="B61" s="21" t="s">
+      <c r="C75" s="44"/>
+    </row>
+    <row r="76" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A76" s="21"/>
+      <c r="B76" s="21" t="s">
         <v>374</v>
       </c>
-      <c r="C61" s="44" t="s">
+      <c r="C76" s="44" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="21"/>
-      <c r="B62" s="48" t="s">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" s="21"/>
+      <c r="B77" s="48" t="s">
         <v>373</v>
       </c>
-      <c r="C62" s="44" t="s">
+      <c r="C77" s="44" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="21"/>
-      <c r="B63" s="21" t="s">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="21"/>
+      <c r="B78" s="21" t="s">
         <v>370</v>
       </c>
-      <c r="C63" s="44" t="s">
+      <c r="C78" s="44" t="s">
         <v>371</v>
       </c>
-      <c r="D63" s="47" t="s">
+      <c r="D78" s="47" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A64" s="21"/>
-      <c r="B64" s="21" t="s">
+    <row r="79" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A79" s="21"/>
+      <c r="B79" s="21" t="s">
         <v>376</v>
       </c>
-      <c r="C64" s="44" t="s">
+      <c r="C79" s="44" t="s">
         <v>375</v>
       </c>
-      <c r="D64" s="44"/>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="46" t="s">
+      <c r="D79" s="44"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="46" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
+    <row r="81" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="B66" s="21" t="s">
+      <c r="B81" s="21" t="s">
+        <v>480</v>
+      </c>
+      <c r="C81" s="44" t="s">
         <v>481</v>
       </c>
-      <c r="C66" s="44" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B67" s="21" t="s">
+    </row>
+    <row r="82" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B82" s="21" t="s">
+        <v>477</v>
+      </c>
+      <c r="C82" s="44" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="B83" s="21" t="s">
+        <v>479</v>
+      </c>
+      <c r="C83" s="68" t="s">
         <v>478</v>
       </c>
-      <c r="C67" s="44" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="316.8" x14ac:dyDescent="0.3">
-      <c r="B68" s="21" t="s">
-        <v>480</v>
-      </c>
-      <c r="C68" s="69" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="13" t="s">
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="13" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B70" s="21" t="s">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B85" s="21" t="s">
         <v>379</v>
       </c>
-      <c r="C70" s="44" t="s">
+      <c r="C85" s="44" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C74" s="43"/>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C75" s="43"/>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C77" s="43"/>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C78" s="43"/>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C79" s="43"/>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C89" s="43"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C90" s="43"/>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C92" s="43"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C93" s="43"/>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C94" s="43"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D45" r:id="rId1" xr:uid="{28B9BCE7-45B7-4868-B75C-CE16E91A776C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -9817,10 +10271,10 @@
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
       <c r="B2" s="51" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
@@ -9869,38 +10323,38 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B11" s="52" t="s">
+        <v>428</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>429</v>
-      </c>
-      <c r="C11" s="49" t="s">
-        <v>435</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B12" s="21" t="s">
+        <v>432</v>
+      </c>
+      <c r="C12" s="49" t="s">
         <v>433</v>
       </c>
-      <c r="C12" s="49" t="s">
-        <v>434</v>
-      </c>
       <c r="D12" s="1" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
+        <v>436</v>
+      </c>
+      <c r="C13" s="49" t="s">
         <v>437</v>
       </c>
-      <c r="C13" s="49" t="s">
-        <v>438</v>
-      </c>
       <c r="D13" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
save 28 08 2026
</commit_message>
<xml_diff>
--- a/4 четверть_26_Cursor.xlsx
+++ b/4 четверть_26_Cursor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42BE39B-21BA-4608-B6AE-2DE9156E7AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504110C9-1F4D-476F-B59E-0D3E0E48DDF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-420" yWindow="-16155" windowWidth="18405" windowHeight="13470" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8040" yWindow="-16080" windowWidth="26445" windowHeight="13470" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Учебные матриалы" sheetId="7" r:id="rId1"/>
@@ -4437,124 +4437,148 @@
 В файле должны быть указаны BEST Practices для построения арзитектуры проекта</t>
   </si>
   <si>
+    <t>Make the critic a habit
+01 When the change is done, open a fresh session (not the one that wrote the code).
+02 Ask for problems, not approval. "Is this good?" gets you a compliment.
+03 Findings only: tell it not to write code. You decide what gets fixed.</t>
+  </si>
+  <si>
+    <t>/create-skill
+Запустить отдельного агента (новый чат) с другой моделью</t>
+  </si>
+  <si>
+    <t>Architecture Decision Records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Только для разработки в команде (не имеет смысла, если один разработчик на проекте)
+</t>
+  </si>
+  <si>
+    <t>Исполнение в строгом соответсвии с правилами кодинга</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Когда хочешь, чтобы </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ИИ выполнил работу строго в соответствии с определенным паттерном</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> проектирования</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Point at an existing module</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+"Structure this like app/Domain/Billing."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Point at a web resource</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+"Read https://stitcher.io/blog/laravel-beyond-crud and structure the new billing"
+"Match the module layout of github.com/spatie/laravel-medialibrary for our uploads rewrite."</t>
+    </r>
+  </si>
+  <si>
     <t>Промпт 1 - CHANGEABILITY
-"Challenge this design for long-term changeability. What change does it make hardest?"
+"Check current changes in git. Challenge this design for long-term changeability. What change does it make hardest?"
 Промпт 2 - COUPLING &amp; OWNERSHIP
 "Find the coupling and ownership problems in this change."
 Промпт 3 - SIMPLER
 "Propose a simpler structure that still meets the requirements. What would we lose?"</t>
-  </si>
-  <si>
-    <t>Make the critic a habit
-01 When the change is done, open a fresh session (not the one that wrote the code).
-02 Ask for problems, not approval. "Is this good?" gets you a compliment.
-03 Findings only: tell it not to write code. You decide what gets fixed.</t>
-  </si>
-  <si>
-    <t>/create-skill
-Запустить отдельного агента (новый чат) с другой моделью</t>
-  </si>
-  <si>
-    <t>Architecture Decision Records</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Только для разработки в команде (не имеет смысла, если один разработчик на проекте)
-</t>
-  </si>
-  <si>
-    <t>Исполнение в строгом соответсвии с правилами кодинга</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Когда хочешь, чтобы </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ИИ выполнил работу строго в соответствии с определенным паттерном</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> проектирования</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Point at an existing module</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-"Structure this like app/Domain/Billing."
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Point at a web resource</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-"Read https://stitcher.io/blog/laravel-beyond-crud and structure the new billing"
-"Match the module layout of github.com/spatie/laravel-medialibrary for our uploads rewrite."</t>
-    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="41" x14ac:knownFonts="1">
+  <fonts count="44" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4950,9 +4974,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -4960,13 +4984,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="29" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4976,7 +5000,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -4989,149 +5013,158 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="26" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="36" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="35" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="41" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="32" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="38" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="41" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="41" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="38" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="38" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -5151,8 +5184,14 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -5160,14 +5199,8 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -9551,7 +9584,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B12" s="22" t="s">
         <v>363</v>
       </c>
@@ -9630,7 +9663,7 @@
       <c r="C19" s="43" t="s">
         <v>406</v>
       </c>
-      <c r="D19" s="55" t="s">
+      <c r="D19" s="77" t="s">
         <v>404</v>
       </c>
     </row>
@@ -9699,7 +9732,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="49"/>
@@ -9707,14 +9740,14 @@
     </row>
     <row r="27" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B27" s="74" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C27" s="49"/>
       <c r="D27" s="49"/>
     </row>
     <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="75" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B28" s="74"/>
       <c r="C28" s="49"/>
@@ -9722,8 +9755,8 @@
     </row>
     <row r="29" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B29" s="74"/>
-      <c r="C29" s="74" t="s">
-        <v>505</v>
+      <c r="C29" s="76" t="s">
+        <v>504</v>
       </c>
       <c r="D29" s="49"/>
     </row>
@@ -9739,7 +9772,7 @@
       <c r="B31" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C31" s="74" t="s">
+      <c r="C31" s="76" t="s">
         <v>494</v>
       </c>
       <c r="D31" s="49"/>
@@ -9754,13 +9787,13 @@
     </row>
     <row r="33" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B33" s="21" t="s">
-        <v>500</v>
-      </c>
-      <c r="C33" s="74" t="s">
+        <v>499</v>
+      </c>
+      <c r="C33" s="78" t="s">
+        <v>505</v>
+      </c>
+      <c r="D33" s="74" t="s">
         <v>498</v>
-      </c>
-      <c r="D33" s="74" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -9773,7 +9806,7 @@
       <c r="D34" s="49"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="61" t="s">
         <v>486</v>
       </c>
       <c r="B35" s="1"/>
@@ -9784,7 +9817,7 @@
       <c r="B36" s="71" t="s">
         <v>488</v>
       </c>
-      <c r="C36" s="74" t="s">
+      <c r="C36" s="78" t="s">
         <v>487</v>
       </c>
       <c r="D36" s="49"/>
@@ -9823,10 +9856,10 @@
     </row>
     <row r="41" spans="1:4" ht="106.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="74" t="s">
+        <v>503</v>
+      </c>
+      <c r="C41" s="74" t="s">
         <v>504</v>
-      </c>
-      <c r="C41" s="74" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>